<commit_message>
flex_scores$gamma limited, update social effects
</commit_message>
<xml_diff>
--- a/inst/ext_data/scenario_parameters.xlsx
+++ b/inst/ext_data/scenario_parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\depmicrosimr\inst\ext_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB320F55-8999-4D73-B5D7-7FAF7F113713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{540E950E-77B5-476B-9CFB-145D3B461001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Description" sheetId="7" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="122">
   <si>
     <t>category</t>
   </si>
@@ -406,6 +406,21 @@
   </si>
   <si>
     <t>not used, social norm model used instead</t>
+  </si>
+  <si>
+    <t>confidence in flexibiity tou (max)</t>
+  </si>
+  <si>
+    <t>pt_certainty_flex_tou_max</t>
+  </si>
+  <si>
+    <t>confidence with zero social reinforcment</t>
+  </si>
+  <si>
+    <t>confidence with full social reinforcement</t>
+  </si>
+  <si>
+    <t>dynamic confidence with zero social refinforement</t>
   </si>
 </sst>
 </file>
@@ -913,7 +928,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C8E1679-ADB0-42D7-8103-5D0EB0C9F50E}">
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -1574,10 +1589,10 @@
         <v>95</v>
       </c>
       <c r="D38">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="E38" t="s">
-        <v>86</v>
+        <v>119</v>
       </c>
       <c r="F38" s="1"/>
     </row>
@@ -1586,32 +1601,36 @@
         <v>86</v>
       </c>
       <c r="B39" t="s">
-        <v>93</v>
+        <v>117</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>96</v>
+        <v>118</v>
       </c>
       <c r="D39">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="E39" t="s">
-        <v>86</v>
+        <v>120</v>
       </c>
       <c r="F39" s="1"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>7</v>
+        <v>86</v>
       </c>
       <c r="B40" t="s">
-        <v>108</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>101</v>
+        <v>93</v>
+      </c>
+      <c r="C40" s="13" t="s">
+        <v>96</v>
       </c>
       <c r="D40">
-        <v>2</v>
-      </c>
+        <v>0.6</v>
+      </c>
+      <c r="E40" t="s">
+        <v>121</v>
+      </c>
+      <c r="F40" s="1"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
@@ -1621,13 +1640,10 @@
         <v>108</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D41">
         <v>2</v>
-      </c>
-      <c r="F41" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
@@ -1635,16 +1651,16 @@
         <v>7</v>
       </c>
       <c r="B42" t="s">
-        <v>75</v>
+        <v>108</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>13</v>
+        <v>102</v>
       </c>
       <c r="D42">
-        <v>0.2</v>
-      </c>
-      <c r="E42" t="s">
-        <v>116</v>
+        <v>2</v>
+      </c>
+      <c r="F42" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -1652,16 +1668,16 @@
         <v>7</v>
       </c>
       <c r="B43" t="s">
-        <v>107</v>
+        <v>75</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D43">
-        <v>0.03</v>
+        <v>0.2</v>
       </c>
       <c r="E43" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
@@ -1669,16 +1685,16 @@
         <v>7</v>
       </c>
       <c r="B44" t="s">
-        <v>6</v>
+        <v>107</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D44">
         <v>0.03</v>
       </c>
       <c r="E44" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
@@ -1686,19 +1702,16 @@
         <v>7</v>
       </c>
       <c r="B45" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="D45">
-        <v>10</v>
+        <v>0.03</v>
       </c>
       <c r="E45" t="s">
-        <v>36</v>
-      </c>
-      <c r="F45" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -1706,15 +1719,35 @@
         <v>7</v>
       </c>
       <c r="B46" t="s">
+        <v>35</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D46">
+        <v>10</v>
+      </c>
+      <c r="E46" t="s">
+        <v>36</v>
+      </c>
+      <c r="F46" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>7</v>
+      </c>
+      <c r="B47" t="s">
         <v>100</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="C47" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D46">
+      <c r="D47">
         <v>0</v>
       </c>
-      <c r="E46" t="s">
+      <c r="E47" t="s">
         <v>113</v>
       </c>
     </row>

</xml_diff>

<commit_message>
hmm states included in set_prices()
</commit_message>
<xml_diff>
--- a/inst/ext_data/scenario_parameters.xlsx
+++ b/inst/ext_data/scenario_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\depmicrosimr\inst\ext_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{540E950E-77B5-476B-9CFB-145D3B461001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2D472AB-18FB-449C-9648-CCABA914138A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="125">
   <si>
     <t>category</t>
   </si>
@@ -421,6 +421,15 @@
   </si>
   <si>
     <t>dynamic confidence with zero social refinforement</t>
+  </si>
+  <si>
+    <t>w_flex</t>
+  </si>
+  <si>
+    <t>unitess</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1-flexibility pass through </t>
   </si>
 </sst>
 </file>
@@ -538,7 +547,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -563,6 +572,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="40% - Accent4" xfId="3" builtinId="43"/>
@@ -928,7 +938,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C8E1679-ADB0-42D7-8103-5D0EB0C9F50E}">
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -1328,23 +1338,20 @@
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>18</v>
-      </c>
-      <c r="B23" t="s">
-        <v>40</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D23">
-        <v>2</v>
+      <c r="A23" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="D23" s="7">
+        <v>0.33333333333333331</v>
       </c>
       <c r="E23" t="s">
-        <v>23</v>
-      </c>
-      <c r="F23" t="s">
-        <v>42</v>
+        <v>123</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -1352,31 +1359,36 @@
         <v>18</v>
       </c>
       <c r="B24" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="D24">
-        <v>130</v>
+        <v>2</v>
       </c>
       <c r="E24" t="s">
-        <v>26</v>
-      </c>
-      <c r="F24" s="1"/>
+        <v>23</v>
+      </c>
+      <c r="F24" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>18</v>
       </c>
       <c r="B25" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D25">
-        <v>215</v>
+        <v>130</v>
+      </c>
+      <c r="E25" t="s">
+        <v>26</v>
       </c>
       <c r="F25" s="1"/>
     </row>
@@ -1385,13 +1397,13 @@
         <v>18</v>
       </c>
       <c r="B26" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D26">
-        <v>265</v>
+        <v>215</v>
       </c>
       <c r="F26" s="1"/>
     </row>
@@ -1400,13 +1412,13 @@
         <v>18</v>
       </c>
       <c r="B27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D27">
-        <v>320</v>
+        <v>265</v>
       </c>
       <c r="F27" s="1"/>
     </row>
@@ -1415,13 +1427,13 @@
         <v>18</v>
       </c>
       <c r="B28" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D28">
-        <v>350</v>
+        <v>320</v>
       </c>
       <c r="F28" s="1"/>
     </row>
@@ -1430,13 +1442,13 @@
         <v>18</v>
       </c>
       <c r="B29" t="s">
-        <v>78</v>
+        <v>34</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>104</v>
+        <v>30</v>
       </c>
       <c r="D29">
-        <v>0</v>
+        <v>350</v>
       </c>
       <c r="F29" s="1"/>
     </row>
@@ -1445,10 +1457,10 @@
         <v>18</v>
       </c>
       <c r="B30" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D30">
         <v>0</v>
@@ -1460,10 +1472,10 @@
         <v>18</v>
       </c>
       <c r="B31" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D31">
         <v>0</v>
@@ -1472,37 +1484,34 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="B32" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>73</v>
+        <v>106</v>
       </c>
       <c r="D32">
-        <v>12</v>
-      </c>
-      <c r="E32" t="s">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="F32" s="1"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>86</v>
+        <v>38</v>
       </c>
       <c r="B33" t="s">
-        <v>89</v>
-      </c>
-      <c r="C33" s="13" t="s">
-        <v>87</v>
+        <v>72</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>73</v>
       </c>
       <c r="D33">
-        <v>0.88</v>
+        <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="F33" s="1"/>
     </row>
@@ -1511,10 +1520,10 @@
         <v>86</v>
       </c>
       <c r="B34" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D34">
         <v>0.88</v>
@@ -1529,13 +1538,13 @@
         <v>86</v>
       </c>
       <c r="B35" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="D35">
-        <v>2.25</v>
+        <v>0.88</v>
       </c>
       <c r="E35" t="s">
         <v>86</v>
@@ -1547,13 +1556,13 @@
         <v>86</v>
       </c>
       <c r="B36" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D36">
-        <v>0.61</v>
+        <v>2.25</v>
       </c>
       <c r="E36" t="s">
         <v>86</v>
@@ -1568,10 +1577,10 @@
         <v>91</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="D37">
-        <v>0.69</v>
+        <v>0.61</v>
       </c>
       <c r="E37" t="s">
         <v>86</v>
@@ -1583,16 +1592,16 @@
         <v>86</v>
       </c>
       <c r="B38" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="D38">
-        <v>0.7</v>
+        <v>0.69</v>
       </c>
       <c r="E38" t="s">
-        <v>119</v>
+        <v>86</v>
       </c>
       <c r="F38" s="1"/>
     </row>
@@ -1601,16 +1610,16 @@
         <v>86</v>
       </c>
       <c r="B39" t="s">
-        <v>117</v>
+        <v>92</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>118</v>
+        <v>95</v>
       </c>
       <c r="D39">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="E39" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F39" s="1"/>
     </row>
@@ -1619,32 +1628,36 @@
         <v>86</v>
       </c>
       <c r="B40" t="s">
-        <v>93</v>
+        <v>117</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>96</v>
+        <v>118</v>
       </c>
       <c r="D40">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="E40" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F40" s="1"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>7</v>
+        <v>86</v>
       </c>
       <c r="B41" t="s">
-        <v>108</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>101</v>
+        <v>93</v>
+      </c>
+      <c r="C41" s="13" t="s">
+        <v>96</v>
       </c>
       <c r="D41">
-        <v>2</v>
-      </c>
+        <v>0.6</v>
+      </c>
+      <c r="E41" t="s">
+        <v>121</v>
+      </c>
+      <c r="F41" s="1"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
@@ -1654,13 +1667,10 @@
         <v>108</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D42">
         <v>2</v>
-      </c>
-      <c r="F42" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -1668,16 +1678,16 @@
         <v>7</v>
       </c>
       <c r="B43" t="s">
-        <v>75</v>
+        <v>108</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>13</v>
+        <v>102</v>
       </c>
       <c r="D43">
-        <v>0.2</v>
-      </c>
-      <c r="E43" t="s">
-        <v>116</v>
+        <v>2</v>
+      </c>
+      <c r="F43" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
@@ -1685,16 +1695,16 @@
         <v>7</v>
       </c>
       <c r="B44" t="s">
-        <v>107</v>
+        <v>75</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D44">
-        <v>0.03</v>
+        <v>0.2</v>
       </c>
       <c r="E44" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
@@ -1702,16 +1712,16 @@
         <v>7</v>
       </c>
       <c r="B45" t="s">
-        <v>6</v>
+        <v>107</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D45">
         <v>0.03</v>
       </c>
       <c r="E45" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -1719,19 +1729,16 @@
         <v>7</v>
       </c>
       <c r="B46" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="D46">
-        <v>10</v>
+        <v>0.03</v>
       </c>
       <c r="E46" t="s">
-        <v>36</v>
-      </c>
-      <c r="F46" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
@@ -1739,15 +1746,35 @@
         <v>7</v>
       </c>
       <c r="B47" t="s">
+        <v>35</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D47">
+        <v>0.01</v>
+      </c>
+      <c r="E47" t="s">
+        <v>36</v>
+      </c>
+      <c r="F47" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>7</v>
+      </c>
+      <c r="B48" t="s">
         <v>100</v>
       </c>
-      <c r="C47" s="3" t="s">
+      <c r="C48" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D47">
+      <c r="D48">
         <v>0</v>
       </c>
-      <c r="E47" t="s">
+      <c r="E48" t="s">
         <v>113</v>
       </c>
     </row>

</xml_diff>

<commit_message>
backflow permitted in prospect model
</commit_message>
<xml_diff>
--- a/inst/ext_data/scenario_parameters.xlsx
+++ b/inst/ext_data/scenario_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\depmicrosimr\inst\ext_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2D472AB-18FB-449C-9648-CCABA914138A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C3FE54B-B6F9-4B7E-B49A-15FEA6F664D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="124">
   <si>
     <t>category</t>
   </si>
@@ -57,9 +57,6 @@
     <t>comment</t>
   </si>
   <si>
-    <t>discount_rate</t>
-  </si>
-  <si>
     <t>calibration</t>
   </si>
   <si>
@@ -76,12 +73,6 @@
   </si>
   <si>
     <t>notes</t>
-  </si>
-  <si>
-    <t>nu.</t>
-  </si>
-  <si>
-    <t>r.</t>
   </si>
   <si>
     <t>introduction time of dynamic pricing</t>
@@ -282,9 +273,6 @@
     <t>12kVA or 12kWh</t>
   </si>
   <si>
-    <t>social factor</t>
-  </si>
-  <si>
     <t>2030 dynamic standing charge</t>
   </si>
   <si>
@@ -405,9 +393,6 @@
     <t>used to handle negative SEM prices</t>
   </si>
   <si>
-    <t>not used, social norm model used instead</t>
-  </si>
-  <si>
     <t>confidence in flexibiity tou (max)</t>
   </si>
   <si>
@@ -430,6 +415,18 @@
   </si>
   <si>
     <t xml:space="preserve">1-flexibility pass through </t>
+  </si>
+  <si>
+    <t>maxmimum allowed value of loss aversion</t>
+  </si>
+  <si>
+    <t>pt_max_loss_aversion</t>
+  </si>
+  <si>
+    <t>minimum allowed value of loss aversion</t>
+  </si>
+  <si>
+    <t>pt_min_loss_aversion</t>
   </si>
 </sst>
 </file>
@@ -547,7 +544,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -572,7 +569,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="40% - Accent4" xfId="3" builtinId="43"/>
@@ -902,32 +898,32 @@
   <sheetData>
     <row r="1" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="14" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>11</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D3" s="5"/>
     </row>
@@ -971,13 +967,13 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D2">
         <v>2026.5</v>
@@ -986,30 +982,30 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D3">
         <v>2021</v>
       </c>
       <c r="F3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D4">
         <v>0.13500000000000001</v>
@@ -1017,13 +1013,13 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D5">
         <v>0.09</v>
@@ -1031,13 +1027,13 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D6">
         <v>0.13500000000000001</v>
@@ -1045,362 +1041,362 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D7">
         <v>0.5</v>
       </c>
       <c r="E7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F7" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D8">
         <v>9.2999999999999999E-2</v>
       </c>
       <c r="E8" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F8" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D9">
         <v>0.15</v>
       </c>
       <c r="E9" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F9" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D10">
         <v>0.2</v>
       </c>
       <c r="E10" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F10" s="1"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D11" s="7">
         <v>0.16838500000000001</v>
       </c>
       <c r="E11" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F11" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D12" s="7">
         <v>7.2419999999999998E-2</v>
       </c>
       <c r="E12" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D13" s="7">
         <v>0.19167500000000001</v>
       </c>
       <c r="E13" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D14">
         <v>0.1981</v>
       </c>
       <c r="E14" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F14" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B15" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D15">
         <v>8.5199999999999998E-2</v>
       </c>
       <c r="E15" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D16">
         <v>0.22550000000000001</v>
       </c>
       <c r="E16" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D17" s="7">
         <v>0.21791000000000002</v>
       </c>
       <c r="E17" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F17" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B18" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D18" s="7">
         <v>9.3720000000000012E-2</v>
       </c>
       <c r="E18" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D19" s="7">
         <v>0.24805000000000002</v>
       </c>
       <c r="E19" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D20" s="7">
         <v>0.25752999999999998</v>
       </c>
       <c r="E20" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F20" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B21" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D21" s="7">
         <v>0.11076</v>
       </c>
       <c r="E21" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D22" s="7">
         <v>0.29315000000000002</v>
       </c>
       <c r="E22" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="B23" s="16" t="s">
-        <v>124</v>
+      <c r="A23" t="s">
+        <v>15</v>
+      </c>
+      <c r="B23" t="s">
+        <v>119</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D23" s="7">
         <v>0.33333333333333331</v>
       </c>
       <c r="E23" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B24" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D24">
         <v>2</v>
       </c>
       <c r="E24" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F24" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B25" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D25">
         <v>130</v>
       </c>
       <c r="E25" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F25" s="1"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B26" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D26">
         <v>215</v>
@@ -1409,13 +1405,13 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B27" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D27">
         <v>265</v>
@@ -1424,13 +1420,13 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B28" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D28">
         <v>320</v>
@@ -1439,13 +1435,13 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B29" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D29">
         <v>350</v>
@@ -1454,13 +1450,13 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B30" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D30">
         <v>0</v>
@@ -1469,13 +1465,13 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B31" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D31">
         <v>0</v>
@@ -1484,13 +1480,13 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B32" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D32">
         <v>0</v>
@@ -1499,283 +1495,279 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B33" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D33">
         <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F33" s="1"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B34" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D34">
         <v>0.88</v>
       </c>
       <c r="E34" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F34" s="1"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
+        <v>82</v>
+      </c>
+      <c r="B35" t="s">
         <v>86</v>
       </c>
-      <c r="B35" t="s">
-        <v>90</v>
-      </c>
       <c r="C35" s="13" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D35">
         <v>0.88</v>
       </c>
       <c r="E35" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F35" s="1"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B36" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D36">
         <v>2.25</v>
       </c>
       <c r="E36" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F36" s="1"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B37" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D37">
         <v>0.61</v>
       </c>
       <c r="E37" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F37" s="1"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B38" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D38">
         <v>0.69</v>
       </c>
       <c r="E38" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F38" s="1"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B39" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="D39">
         <v>0.7</v>
       </c>
       <c r="E39" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="F39" s="1"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B40" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="D40">
         <v>0.9</v>
       </c>
       <c r="E40" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="F40" s="1"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B41" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D41">
         <v>0.6</v>
       </c>
       <c r="E41" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="F41" s="1"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
       <c r="B42" t="s">
-        <v>108</v>
-      </c>
-      <c r="C42" s="3" t="s">
-        <v>101</v>
+        <v>120</v>
+      </c>
+      <c r="C42" s="13" t="s">
+        <v>121</v>
       </c>
       <c r="D42">
-        <v>2</v>
-      </c>
+        <v>3.25</v>
+      </c>
+      <c r="F42" s="1"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
       <c r="B43" t="s">
-        <v>108</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>102</v>
+        <v>122</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>123</v>
       </c>
       <c r="D43">
-        <v>2</v>
-      </c>
-      <c r="F43" t="s">
-        <v>103</v>
-      </c>
+        <v>1.25</v>
+      </c>
+      <c r="F43" s="1"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B44" t="s">
-        <v>75</v>
+        <v>104</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>13</v>
+        <v>97</v>
       </c>
       <c r="D44">
-        <v>0.2</v>
-      </c>
-      <c r="E44" t="s">
-        <v>116</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B45" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>8</v>
+        <v>98</v>
       </c>
       <c r="D45">
-        <v>0.03</v>
-      </c>
-      <c r="E45" t="s">
-        <v>114</v>
+        <v>2</v>
+      </c>
+      <c r="F45" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
+        <v>6</v>
+      </c>
+      <c r="B46" t="s">
+        <v>103</v>
+      </c>
+      <c r="C46" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B46" t="s">
-        <v>6</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>14</v>
-      </c>
       <c r="D46">
-        <v>0.03</v>
+        <v>2.7E-2</v>
       </c>
       <c r="E46" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B47" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D47">
         <v>0.01</v>
       </c>
       <c r="E47" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F47" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B48" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D48">
         <v>0</v>
       </c>
       <c r="E48" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
heterogeneous loss aversion added
</commit_message>
<xml_diff>
--- a/inst/ext_data/scenario_parameters.xlsx
+++ b/inst/ext_data/scenario_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\depmicrosimr\inst\ext_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C3FE54B-B6F9-4B7E-B49A-15FEA6F664D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF129154-3805-48BF-A62A-3A1448A1D60A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="127">
   <si>
     <t>category</t>
   </si>
@@ -369,9 +369,6 @@
     <t>inertia param (p_rate)</t>
   </si>
   <si>
-    <t xml:space="preserve">beta distribution </t>
-  </si>
-  <si>
     <t>BASE</t>
   </si>
   <si>
@@ -427,6 +424,18 @@
   </si>
   <si>
     <t>pt_min_loss_aversion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flex score beta distribution </t>
+  </si>
+  <si>
+    <t xml:space="preserve">flex beta distribution </t>
+  </si>
+  <si>
+    <t>loss_alpha.</t>
+  </si>
+  <si>
+    <t>loss_beta.</t>
   </si>
 </sst>
 </file>
@@ -898,7 +907,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -917,13 +926,13 @@
     </row>
     <row r="3" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="C3" s="5" t="s">
         <v>106</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>107</v>
       </c>
       <c r="D3" s="5"/>
     </row>
@@ -934,7 +943,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C8E1679-ADB0-42D7-8103-5D0EB0C9F50E}">
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -1338,16 +1347,16 @@
         <v>15</v>
       </c>
       <c r="B23" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D23" s="7">
         <v>0.33333333333333331</v>
       </c>
       <c r="E23" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -1615,7 +1624,7 @@
         <v>0.7</v>
       </c>
       <c r="E39" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F39" s="1"/>
     </row>
@@ -1624,16 +1633,16 @@
         <v>82</v>
       </c>
       <c r="B40" t="s">
+        <v>111</v>
+      </c>
+      <c r="C40" s="13" t="s">
         <v>112</v>
-      </c>
-      <c r="C40" s="13" t="s">
-        <v>113</v>
       </c>
       <c r="D40">
         <v>0.9</v>
       </c>
       <c r="E40" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F40" s="1"/>
     </row>
@@ -1651,7 +1660,7 @@
         <v>0.6</v>
       </c>
       <c r="E41" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F41" s="1"/>
     </row>
@@ -1660,13 +1669,13 @@
         <v>82</v>
       </c>
       <c r="B42" t="s">
+        <v>119</v>
+      </c>
+      <c r="C42" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="C42" s="13" t="s">
-        <v>121</v>
-      </c>
       <c r="D42">
-        <v>3.25</v>
+        <v>4.25</v>
       </c>
       <c r="F42" s="1"/>
     </row>
@@ -1675,10 +1684,10 @@
         <v>82</v>
       </c>
       <c r="B43" t="s">
+        <v>121</v>
+      </c>
+      <c r="C43" s="13" t="s">
         <v>122</v>
-      </c>
-      <c r="C43" s="13" t="s">
-        <v>123</v>
       </c>
       <c r="D43">
         <v>1.25</v>
@@ -1690,7 +1699,7 @@
         <v>6</v>
       </c>
       <c r="B44" t="s">
-        <v>104</v>
+        <v>123</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>97</v>
@@ -1704,7 +1713,7 @@
         <v>6</v>
       </c>
       <c r="B45" t="s">
-        <v>104</v>
+        <v>124</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>98</v>
@@ -1721,16 +1730,13 @@
         <v>6</v>
       </c>
       <c r="B46" t="s">
-        <v>103</v>
+        <v>123</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>7</v>
+        <v>125</v>
       </c>
       <c r="D46">
-        <v>2.7E-2</v>
-      </c>
-      <c r="E46" t="s">
-        <v>110</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
@@ -1738,19 +1744,16 @@
         <v>6</v>
       </c>
       <c r="B47" t="s">
-        <v>32</v>
+        <v>124</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>34</v>
+        <v>126</v>
       </c>
       <c r="D47">
-        <v>0.01</v>
-      </c>
-      <c r="E47" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="F47" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -1758,16 +1761,53 @@
         <v>6</v>
       </c>
       <c r="B48" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="D48">
-        <v>0</v>
+        <v>2.7E-2</v>
       </c>
       <c r="E48" t="s">
         <v>109</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>6</v>
+      </c>
+      <c r="B49" t="s">
+        <v>32</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D49">
+        <v>0.01</v>
+      </c>
+      <c r="E49" t="s">
+        <v>33</v>
+      </c>
+      <c r="F49" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>6</v>
+      </c>
+      <c r="B50" t="s">
+        <v>96</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+      <c r="E50" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sem_prices() bug; shock added
</commit_message>
<xml_diff>
--- a/inst/ext_data/scenario_parameters.xlsx
+++ b/inst/ext_data/scenario_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\depmicrosimr\inst\ext_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF129154-3805-48BF-A62A-3A1448A1D60A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{773631BE-9871-4026-89D4-85894BEECF94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -291,18 +291,12 @@
     <t>trend price at end of 2025</t>
   </si>
   <si>
-    <t>CU 2026 dynamic price cap</t>
-  </si>
-  <si>
     <t>dynamic_cap</t>
   </si>
   <si>
     <t>CRU cap in 2026/ Assumed to scale with sem trend price</t>
   </si>
   <si>
-    <t>trend wholesale price</t>
-  </si>
-  <si>
     <t>prospect theory</t>
   </si>
   <si>
@@ -436,6 +430,12 @@
   </si>
   <si>
     <t>loss_beta.</t>
+  </si>
+  <si>
+    <t>trend wholesale price at end of 2030</t>
+  </si>
+  <si>
+    <t>CRU 2026 dynamic price cap</t>
   </si>
 </sst>
 </file>
@@ -907,7 +907,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="14" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -926,13 +926,13 @@
     </row>
     <row r="3" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>104</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>106</v>
       </c>
       <c r="D3" s="5"/>
     </row>
@@ -1053,10 +1053,10 @@
         <v>13</v>
       </c>
       <c r="B7" t="s">
+        <v>126</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>78</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>79</v>
       </c>
       <c r="D7">
         <v>0.5</v>
@@ -1065,7 +1065,7 @@
         <v>16</v>
       </c>
       <c r="F7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -1105,7 +1105,7 @@
         <v>16</v>
       </c>
       <c r="F9" t="s">
-        <v>81</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -1347,16 +1347,16 @@
         <v>15</v>
       </c>
       <c r="B23" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D23" s="7">
         <v>0.33333333333333331</v>
       </c>
       <c r="E23" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -1465,7 +1465,7 @@
         <v>74</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D30">
         <v>0</v>
@@ -1480,7 +1480,7 @@
         <v>72</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D31">
         <v>0</v>
@@ -1495,7 +1495,7 @@
         <v>73</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D32">
         <v>0</v>
@@ -1522,157 +1522,157 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B34" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D34">
         <v>0.88</v>
       </c>
       <c r="E34" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F34" s="1"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
+        <v>80</v>
+      </c>
+      <c r="B35" t="s">
+        <v>84</v>
+      </c>
+      <c r="C35" s="13" t="s">
         <v>82</v>
-      </c>
-      <c r="B35" t="s">
-        <v>86</v>
-      </c>
-      <c r="C35" s="13" t="s">
-        <v>84</v>
       </c>
       <c r="D35">
         <v>0.88</v>
       </c>
       <c r="E35" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F35" s="1"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B36" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D36">
         <v>2.25</v>
       </c>
       <c r="E36" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F36" s="1"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B37" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D37">
         <v>0.61</v>
       </c>
       <c r="E37" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F37" s="1"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B38" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D38">
         <v>0.69</v>
       </c>
       <c r="E38" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F38" s="1"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B39" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D39">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="E39" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F39" s="1"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B40" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C40" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="D40">
+        <v>0.75</v>
+      </c>
+      <c r="E40" t="s">
         <v>112</v>
-      </c>
-      <c r="D40">
-        <v>0.9</v>
-      </c>
-      <c r="E40" t="s">
-        <v>114</v>
       </c>
       <c r="F40" s="1"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D41">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="E41" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F41" s="1"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B42" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D42">
         <v>4.25</v>
@@ -1681,13 +1681,13 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B43" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D43">
         <v>1.25</v>
@@ -1699,10 +1699,10 @@
         <v>6</v>
       </c>
       <c r="B44" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D44">
         <v>2</v>
@@ -1713,16 +1713,16 @@
         <v>6</v>
       </c>
       <c r="B45" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D45">
         <v>2</v>
       </c>
       <c r="F45" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -1730,10 +1730,10 @@
         <v>6</v>
       </c>
       <c r="B46" t="s">
+        <v>121</v>
+      </c>
+      <c r="C46" s="3" t="s">
         <v>123</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>125</v>
       </c>
       <c r="D46">
         <v>2</v>
@@ -1744,16 +1744,16 @@
         <v>6</v>
       </c>
       <c r="B47" t="s">
+        <v>122</v>
+      </c>
+      <c r="C47" s="3" t="s">
         <v>124</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>126</v>
       </c>
       <c r="D47">
         <v>4</v>
       </c>
       <c r="F47" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -1761,7 +1761,7 @@
         <v>6</v>
       </c>
       <c r="B48" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>7</v>
@@ -1770,7 +1770,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="E48" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -1790,7 +1790,7 @@
         <v>33</v>
       </c>
       <c r="F49" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -1798,7 +1798,7 @@
         <v>6</v>
       </c>
       <c r="B50" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>36</v>
@@ -1807,7 +1807,7 @@
         <v>0</v>
       </c>
       <c r="E50" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
full behavioural cost + prospect
</commit_message>
<xml_diff>
--- a/inst/ext_data/scenario_parameters.xlsx
+++ b/inst/ext_data/scenario_parameters.xlsx
@@ -8,13 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\depmicrosimr\inst\ext_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{773631BE-9871-4026-89D4-85894BEECF94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5C5828F-A711-4379-90E9-2DAE1D237F79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Description" sheetId="7" r:id="rId1"/>
     <sheet name="Base" sheetId="16" r:id="rId2"/>
+    <sheet name="LDSC" sheetId="17" r:id="rId3"/>
+    <sheet name="HDSC" sheetId="18" r:id="rId4"/>
+    <sheet name="LowPrice" sheetId="20" r:id="rId5"/>
+    <sheet name="HighPrice" sheetId="19" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="144">
   <si>
     <t>category</t>
   </si>
@@ -67,9 +71,6 @@
   </si>
   <si>
     <t>tag</t>
-  </si>
-  <si>
-    <t>name</t>
   </si>
   <si>
     <t>notes</t>
@@ -372,9 +373,6 @@
     <t>More or less the current situation except that the standing charge for all tariff plans are assumed to be the same</t>
   </si>
   <si>
-    <t>depmicromsimr scenario description</t>
-  </si>
-  <si>
     <t>not used</t>
   </si>
   <si>
@@ -436,6 +434,83 @@
   </si>
   <si>
     <t>CRU 2026 dynamic price cap</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>LDSC</t>
+  </si>
+  <si>
+    <t>HDSC</t>
+  </si>
+  <si>
+    <t>High dynamic standing charge</t>
+  </si>
+  <si>
+    <t>Low dynamic standing charge</t>
+  </si>
+  <si>
+    <t>LowPrice</t>
+  </si>
+  <si>
+    <t>HighPrice</t>
+  </si>
+  <si>
+    <r>
+      <t>2030 0.1€/kWh 2040 0.1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>€</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>/kWh</t>
+    </r>
+  </si>
+  <si>
+    <t>2030 0.2€/kWh 2040 0.3€/kWh</t>
+  </si>
+  <si>
+    <t>-75 €</t>
+  </si>
+  <si>
+    <t>+75 €</t>
+  </si>
+  <si>
+    <t>NoToU</t>
+  </si>
+  <si>
+    <t>remove ToU in 2030</t>
+  </si>
+  <si>
+    <t>Battery</t>
+  </si>
+  <si>
+    <t>high battery uptake</t>
+  </si>
+  <si>
+    <t>reduce phi and increase tau so that households become more flexible at each time step</t>
+  </si>
+  <si>
+    <t>random battery uptake model means that flex_score distribution become right-skewed</t>
+  </si>
+  <si>
+    <t>depmicromsimr scenario descriptions</t>
+  </si>
+  <si>
+    <t>label</t>
   </si>
 </sst>
 </file>
@@ -445,7 +520,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -494,6 +569,18 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -553,7 +640,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -574,9 +661,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -895,10 +990,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2536B528-ACE0-4AEE-80FE-2144BA4A4410}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.44140625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="26.44140625" style="17" customWidth="1"/>
     <col min="2" max="2" width="37.77734375" style="2" customWidth="1"/>
     <col min="3" max="3" width="43.33203125" style="2" customWidth="1"/>
     <col min="4" max="4" width="33.21875" style="2" customWidth="1"/>
@@ -906,13 +1001,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="14" t="s">
-        <v>105</v>
+      <c r="A1" s="16" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>10</v>
+        <v>143</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>9</v>
@@ -921,20 +1016,80 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="C3" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>104</v>
-      </c>
       <c r="D3" s="5"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="17" t="s">
+        <v>126</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="17" t="s">
+        <v>127</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>141</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -976,13 +1131,13 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>14</v>
       </c>
       <c r="D2">
         <v>2026.5</v>
@@ -991,30 +1146,30 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>17</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>18</v>
       </c>
       <c r="D3">
         <v>2021</v>
       </c>
       <c r="F3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D4">
         <v>0.13500000000000001</v>
@@ -1022,13 +1177,13 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D5">
         <v>0.09</v>
@@ -1036,13 +1191,13 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>67</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>68</v>
       </c>
       <c r="D6">
         <v>0.13500000000000001</v>
@@ -1050,362 +1205,362 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D7">
         <v>0.5</v>
       </c>
       <c r="E7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D8">
         <v>9.2999999999999999E-2</v>
       </c>
       <c r="E8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D9">
         <v>0.15</v>
       </c>
       <c r="E9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F9" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D10">
         <v>0.2</v>
       </c>
       <c r="E10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F10" s="1"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B11" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="D11" s="7">
         <v>0.16838500000000001</v>
       </c>
       <c r="E11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D12" s="7">
         <v>7.2419999999999998E-2</v>
       </c>
       <c r="E12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D13" s="7">
         <v>0.19167500000000001</v>
       </c>
       <c r="E13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D14">
         <v>0.1981</v>
       </c>
       <c r="E14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F14" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D15">
         <v>8.5199999999999998E-2</v>
       </c>
       <c r="E15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D16">
         <v>0.22550000000000001</v>
       </c>
       <c r="E16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D17" s="7">
         <v>0.21791000000000002</v>
       </c>
       <c r="E17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D18" s="7">
         <v>9.3720000000000012E-2</v>
       </c>
       <c r="E18" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D19" s="7">
         <v>0.24805000000000002</v>
       </c>
       <c r="E19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D20" s="7">
         <v>0.25752999999999998</v>
       </c>
       <c r="E20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B21" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D21" s="7">
         <v>0.11076</v>
       </c>
       <c r="E21" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D22" s="7">
         <v>0.29315000000000002</v>
       </c>
       <c r="E22" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B23" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D23" s="7">
         <v>0.33333333333333331</v>
       </c>
       <c r="E23" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B24" t="s">
+        <v>36</v>
+      </c>
+      <c r="C24" s="6" t="s">
         <v>37</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>38</v>
       </c>
       <c r="D24">
         <v>2</v>
       </c>
       <c r="E24" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F24" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B25" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="D25">
         <v>130</v>
       </c>
       <c r="E25" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F25" s="1"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B26" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D26">
         <v>215</v>
@@ -1414,13 +1569,13 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B27" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D27">
         <v>265</v>
@@ -1429,13 +1584,13 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B28" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D28">
         <v>320</v>
@@ -1444,13 +1599,13 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D29">
         <v>350</v>
@@ -1459,13 +1614,13 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B30" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D30">
         <v>0</v>
@@ -1474,13 +1629,13 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D31">
         <v>0</v>
@@ -1489,13 +1644,13 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B32" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D32">
         <v>0</v>
@@ -1504,175 +1659,175 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B33" t="s">
+        <v>68</v>
+      </c>
+      <c r="C33" s="6" t="s">
         <v>69</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>70</v>
       </c>
       <c r="D33">
         <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F33" s="1"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>79</v>
+      </c>
+      <c r="B34" t="s">
+        <v>82</v>
+      </c>
+      <c r="C34" s="13" t="s">
         <v>80</v>
-      </c>
-      <c r="B34" t="s">
-        <v>83</v>
-      </c>
-      <c r="C34" s="13" t="s">
-        <v>81</v>
       </c>
       <c r="D34">
         <v>0.88</v>
       </c>
       <c r="E34" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F34" s="1"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B35" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D35">
         <v>0.88</v>
       </c>
       <c r="E35" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F35" s="1"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B36" t="s">
+        <v>90</v>
+      </c>
+      <c r="C36" s="13" t="s">
         <v>91</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>92</v>
       </c>
       <c r="D36">
         <v>2.25</v>
       </c>
       <c r="E36" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F36" s="1"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B37" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D37">
         <v>0.61</v>
       </c>
       <c r="E37" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F37" s="1"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B38" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D38">
         <v>0.69</v>
       </c>
       <c r="E38" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F38" s="1"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B39" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D39">
-        <v>0.5</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="E39" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F39" s="1"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B40" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D40">
         <v>0.75</v>
       </c>
       <c r="E40" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F40" s="1"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B41" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D41">
         <v>0.4</v>
       </c>
       <c r="E41" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F41" s="1"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B42" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D42">
         <v>4.25</v>
@@ -1681,13 +1836,13 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B43" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D43">
         <v>1.25</v>
@@ -1699,10 +1854,10 @@
         <v>6</v>
       </c>
       <c r="B44" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D44">
         <v>2</v>
@@ -1713,16 +1868,16 @@
         <v>6</v>
       </c>
       <c r="B45" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D45">
         <v>2</v>
       </c>
       <c r="F45" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -1730,10 +1885,10 @@
         <v>6</v>
       </c>
       <c r="B46" t="s">
+        <v>119</v>
+      </c>
+      <c r="C46" s="3" t="s">
         <v>121</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>123</v>
       </c>
       <c r="D46">
         <v>2</v>
@@ -1744,16 +1899,16 @@
         <v>6</v>
       </c>
       <c r="B47" t="s">
+        <v>120</v>
+      </c>
+      <c r="C47" s="3" t="s">
         <v>122</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>124</v>
       </c>
       <c r="D47">
         <v>4</v>
       </c>
       <c r="F47" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -1761,7 +1916,7 @@
         <v>6</v>
       </c>
       <c r="B48" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>7</v>
@@ -1770,7 +1925,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="E48" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -1778,19 +1933,19 @@
         <v>6</v>
       </c>
       <c r="B49" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D49">
         <v>0.01</v>
       </c>
       <c r="E49" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F49" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -1798,19 +1953,61 @@
         <v>6</v>
       </c>
       <c r="B50" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D50">
         <v>0</v>
       </c>
       <c r="E50" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFE7130B-2B6C-40C3-A565-474237859EF4}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A8FF8BC-953A-45D1-A042-B3C357C0F4A0}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEB88E62-7607-4F45-BA84-25687CEF5DCD}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{637651EF-BBD1-4820-B575-600BCC8F4568}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
flat & tou tariffs based on rolling average of previous year dynamic
</commit_message>
<xml_diff>
--- a/inst/ext_data/scenario_parameters.xlsx
+++ b/inst/ext_data/scenario_parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\depmicrosimr\inst\ext_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5C5828F-A711-4379-90E9-2DAE1D237F79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{769B1355-A5B3-444C-A8B9-9A74788CCD3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Description" sheetId="7" r:id="rId1"/>
@@ -1254,7 +1254,7 @@
         <v>60</v>
       </c>
       <c r="D9">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="E9" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
q_dyn and q_tou and q_tou_old fixes
</commit_message>
<xml_diff>
--- a/inst/ext_data/scenario_parameters.xlsx
+++ b/inst/ext_data/scenario_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\depmicrosimr\inst\ext_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F99047F-0034-423F-880E-C4902B7D32CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE9B50A3-7774-4E1C-A436-4778CD88B0F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1628,7 +1628,7 @@
         <v>96</v>
       </c>
       <c r="D30">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F30" s="1"/>
     </row>
@@ -1643,7 +1643,7 @@
         <v>97</v>
       </c>
       <c r="D31">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F31" s="1"/>
     </row>
@@ -1658,7 +1658,7 @@
         <v>98</v>
       </c>
       <c r="D32">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F32" s="1"/>
     </row>

</xml_diff>

<commit_message>
dynamic awareness yeartime added
</commit_message>
<xml_diff>
--- a/inst/ext_data/scenario_parameters.xlsx
+++ b/inst/ext_data/scenario_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\depmicrosimr\inst\ext_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE9B50A3-7774-4E1C-A436-4778CD88B0F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8C65864-3899-4303-8278-88DAB3ED7743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="148">
   <si>
     <t>category</t>
   </si>
@@ -514,6 +514,15 @@
   </si>
   <si>
     <t>parameters defined for "full" scenario (provisionally)</t>
+  </si>
+  <si>
+    <t>dyn_aware_year</t>
+  </si>
+  <si>
+    <t>year of full awareness of dep</t>
+  </si>
+  <si>
+    <t>year time at which awareness of dynamic pricing is universal. Must be &gt; 2026.5.</t>
   </si>
 </sst>
 </file>
@@ -1103,7 +1112,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C8E1679-ADB0-42D7-8103-5D0EB0C9F50E}">
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -1968,6 +1977,23 @@
       </c>
       <c r="E50" t="s">
         <v>143</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>6</v>
+      </c>
+      <c r="B51" t="s">
+        <v>146</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="D51">
+        <v>2030</v>
+      </c>
+      <c r="E51" t="s">
+        <v>147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added dyn_aware to initialise_agents
</commit_message>
<xml_diff>
--- a/inst/ext_data/scenario_parameters.xlsx
+++ b/inst/ext_data/scenario_parameters.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\depmicrosimr\inst\ext_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8C65864-3899-4303-8278-88DAB3ED7743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7E7C3F1-CF76-4FA1-8E79-790198C1BDE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Description" sheetId="7" r:id="rId1"/>
     <sheet name="Base" sheetId="16" r:id="rId2"/>
-    <sheet name="LDSC" sheetId="17" r:id="rId3"/>
-    <sheet name="HDSC" sheetId="18" r:id="rId4"/>
+    <sheet name="EDSC" sheetId="17" r:id="rId3"/>
+    <sheet name="LDSC" sheetId="18" r:id="rId4"/>
     <sheet name="LowPrice" sheetId="20" r:id="rId5"/>
     <sheet name="HighPrice" sheetId="19" r:id="rId6"/>
   </sheets>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1025" uniqueCount="149">
   <si>
     <t>category</t>
   </si>
@@ -430,13 +430,7 @@
     <t>CRU 2026 dynamic price cap</t>
   </si>
   <si>
-    <t>H</t>
-  </si>
-  <si>
     <t>LDSC</t>
-  </si>
-  <si>
-    <t>HDSC</t>
   </si>
   <si>
     <t>High dynamic standing charge</t>
@@ -523,6 +517,15 @@
   </si>
   <si>
     <t>year time at which awareness of dynamic pricing is universal. Must be &gt; 2026.5.</t>
+  </si>
+  <si>
+    <t>loss averssion beta distribution alpha</t>
+  </si>
+  <si>
+    <t>loss averssion beta distribution beta</t>
+  </si>
+  <si>
+    <t>EDSC</t>
   </si>
 </sst>
 </file>
@@ -1014,12 +1017,12 @@
   <sheetData>
     <row r="1" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="16" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>9</v>
@@ -1042,67 +1045,67 @@
         <v>102</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="17" t="s">
-        <v>124</v>
+        <v>148</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="17" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="17" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="17" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="17" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
+        <v>134</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>137</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -1790,7 +1793,7 @@
         <v>87</v>
       </c>
       <c r="D39">
-        <v>0.75</v>
+        <v>0.7</v>
       </c>
       <c r="E39" t="s">
         <v>107</v>
@@ -1826,7 +1829,7 @@
         <v>88</v>
       </c>
       <c r="D41">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="E41" t="s">
         <v>109</v>
@@ -1936,7 +1939,7 @@
         <v>7</v>
       </c>
       <c r="D48">
-        <v>2.7E-2</v>
+        <v>0.03</v>
       </c>
       <c r="E48" t="s">
         <v>103</v>
@@ -1970,13 +1973,13 @@
         <v>92</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D50">
         <v>0.3</v>
       </c>
       <c r="E50" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
@@ -1984,16 +1987,16 @@
         <v>6</v>
       </c>
       <c r="B51" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D51">
         <v>2030</v>
       </c>
       <c r="E51" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -2003,21 +2006,1779 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFE7130B-2B6C-40C3-A565-474237859EF4}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="2" max="2" width="41.88671875" customWidth="1"/>
+    <col min="3" max="3" width="55" customWidth="1"/>
+    <col min="4" max="4" width="16.5546875" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" customWidth="1"/>
+    <col min="6" max="6" width="22.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2">
+        <v>2026.5</v>
+      </c>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3">
+        <v>2021</v>
+      </c>
+      <c r="F3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="D4">
+        <v>0.13500000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="D5">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6">
+        <v>0.13500000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>122</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D7">
+        <v>0.5</v>
+      </c>
+      <c r="E7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="D8">
+        <v>9.2999999999999999E-2</v>
+      </c>
+      <c r="E8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9">
+        <v>0.13</v>
+      </c>
+      <c r="E9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10">
+        <v>0.2</v>
+      </c>
+      <c r="E10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" s="7">
+        <v>0.16838500000000001</v>
+      </c>
+      <c r="E11" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" s="7">
+        <v>7.2419999999999998E-2</v>
+      </c>
+      <c r="E12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="7">
+        <v>0.19167500000000001</v>
+      </c>
+      <c r="E13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="D14">
+        <v>0.1981</v>
+      </c>
+      <c r="E14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15">
+        <v>8.5199999999999998E-2</v>
+      </c>
+      <c r="E15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D16">
+        <v>0.22550000000000001</v>
+      </c>
+      <c r="E16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="7">
+        <v>0.21791000000000002</v>
+      </c>
+      <c r="E17" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" s="7">
+        <v>9.3720000000000012E-2</v>
+      </c>
+      <c r="E18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="7">
+        <v>0.24805000000000002</v>
+      </c>
+      <c r="E19" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D20" s="7">
+        <v>0.25752999999999998</v>
+      </c>
+      <c r="E20" t="s">
+        <v>15</v>
+      </c>
+      <c r="F20" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D21" s="7">
+        <v>0.11076</v>
+      </c>
+      <c r="E21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D22" s="7">
+        <v>0.29315000000000002</v>
+      </c>
+      <c r="E22" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>14</v>
+      </c>
+      <c r="B23" t="s">
+        <v>112</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="D23" s="7">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="E23" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>14</v>
+      </c>
+      <c r="B24" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D24">
+        <v>2</v>
+      </c>
+      <c r="E24" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B25" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D25">
+        <v>130</v>
+      </c>
+      <c r="E25" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25" s="1"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B26" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D26">
+        <v>215</v>
+      </c>
+      <c r="F26" s="1"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B27" t="s">
+        <v>28</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D27">
+        <v>265</v>
+      </c>
+      <c r="F27" s="1"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D28">
+        <v>320</v>
+      </c>
+      <c r="F28" s="1"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>14</v>
+      </c>
+      <c r="B29" t="s">
+        <v>30</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D29">
+        <v>350</v>
+      </c>
+      <c r="F29" s="1"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>14</v>
+      </c>
+      <c r="B30" t="s">
+        <v>72</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D30">
+        <v>75</v>
+      </c>
+      <c r="F30" s="1"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>14</v>
+      </c>
+      <c r="B31" t="s">
+        <v>70</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="F31" s="1"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>14</v>
+      </c>
+      <c r="B32" t="s">
+        <v>71</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="F32" s="1"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>34</v>
+      </c>
+      <c r="B33" t="s">
+        <v>67</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D33">
+        <v>12</v>
+      </c>
+      <c r="E33" t="s">
+        <v>69</v>
+      </c>
+      <c r="F33" s="1"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>78</v>
+      </c>
+      <c r="B34" t="s">
+        <v>81</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="D34">
+        <v>0.88</v>
+      </c>
+      <c r="E34" t="s">
+        <v>78</v>
+      </c>
+      <c r="F34" s="1"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>78</v>
+      </c>
+      <c r="B35" t="s">
+        <v>82</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="D35">
+        <v>0.88</v>
+      </c>
+      <c r="E35" t="s">
+        <v>78</v>
+      </c>
+      <c r="F35" s="1"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>78</v>
+      </c>
+      <c r="B36" t="s">
+        <v>89</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="D36">
+        <v>2.25</v>
+      </c>
+      <c r="E36" t="s">
+        <v>78</v>
+      </c>
+      <c r="F36" s="1"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>78</v>
+      </c>
+      <c r="B37" t="s">
+        <v>83</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D37">
+        <v>0.61</v>
+      </c>
+      <c r="E37" t="s">
+        <v>78</v>
+      </c>
+      <c r="F37" s="1"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>78</v>
+      </c>
+      <c r="B38" t="s">
+        <v>83</v>
+      </c>
+      <c r="C38" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D38">
+        <v>0.69</v>
+      </c>
+      <c r="E38" t="s">
+        <v>78</v>
+      </c>
+      <c r="F38" s="1"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>78</v>
+      </c>
+      <c r="B39" t="s">
+        <v>84</v>
+      </c>
+      <c r="C39" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="D39">
+        <v>0.7</v>
+      </c>
+      <c r="E39" t="s">
+        <v>107</v>
+      </c>
+      <c r="F39" s="1"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>78</v>
+      </c>
+      <c r="B40" t="s">
+        <v>105</v>
+      </c>
+      <c r="C40" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="D40">
+        <v>0.9</v>
+      </c>
+      <c r="E40" t="s">
+        <v>108</v>
+      </c>
+      <c r="F40" s="1"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>78</v>
+      </c>
+      <c r="B41" t="s">
+        <v>85</v>
+      </c>
+      <c r="C41" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="D41">
+        <v>0.4</v>
+      </c>
+      <c r="E41" t="s">
+        <v>109</v>
+      </c>
+      <c r="F41" s="1"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>78</v>
+      </c>
+      <c r="B42" t="s">
+        <v>113</v>
+      </c>
+      <c r="C42" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="D42">
+        <v>4.25</v>
+      </c>
+      <c r="F42" s="1"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>78</v>
+      </c>
+      <c r="B43" t="s">
+        <v>115</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="D43">
+        <v>1.25</v>
+      </c>
+      <c r="F43" s="1"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>6</v>
+      </c>
+      <c r="B44" t="s">
+        <v>117</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D44">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>6</v>
+      </c>
+      <c r="B45" t="s">
+        <v>118</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="D45">
+        <v>2</v>
+      </c>
+      <c r="F45" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>6</v>
+      </c>
+      <c r="B46" t="s">
+        <v>146</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="D46">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>6</v>
+      </c>
+      <c r="B47" t="s">
+        <v>147</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D47">
+        <v>4</v>
+      </c>
+      <c r="F47" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>6</v>
+      </c>
+      <c r="B48" t="s">
+        <v>99</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>0.03</v>
+      </c>
+      <c r="E48" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>6</v>
+      </c>
+      <c r="B49" t="s">
+        <v>31</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D49">
+        <v>0.01</v>
+      </c>
+      <c r="E49" t="s">
+        <v>32</v>
+      </c>
+      <c r="F49" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>6</v>
+      </c>
+      <c r="B50" t="s">
+        <v>92</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D50">
+        <v>0.3</v>
+      </c>
+      <c r="E50" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>6</v>
+      </c>
+      <c r="B51" t="s">
+        <v>144</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D51">
+        <v>2030</v>
+      </c>
+      <c r="E51" t="s">
+        <v>145</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A8FF8BC-953A-45D1-A042-B3C357C0F4A0}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="2" max="2" width="41.88671875" customWidth="1"/>
+    <col min="3" max="3" width="55" customWidth="1"/>
+    <col min="4" max="4" width="16.5546875" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" customWidth="1"/>
+    <col min="6" max="6" width="22.5546875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>123</v>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2">
+        <v>2026.5</v>
+      </c>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3">
+        <v>2021</v>
+      </c>
+      <c r="F3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="D4">
+        <v>0.13500000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="D5">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6">
+        <v>0.13500000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>122</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D7">
+        <v>0.5</v>
+      </c>
+      <c r="E7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="D8">
+        <v>9.2999999999999999E-2</v>
+      </c>
+      <c r="E8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9">
+        <v>0.13</v>
+      </c>
+      <c r="E9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10">
+        <v>0.2</v>
+      </c>
+      <c r="E10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" s="7">
+        <v>0.16838500000000001</v>
+      </c>
+      <c r="E11" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" s="7">
+        <v>7.2419999999999998E-2</v>
+      </c>
+      <c r="E12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="7">
+        <v>0.19167500000000001</v>
+      </c>
+      <c r="E13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="D14">
+        <v>0.1981</v>
+      </c>
+      <c r="E14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15">
+        <v>8.5199999999999998E-2</v>
+      </c>
+      <c r="E15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D16">
+        <v>0.22550000000000001</v>
+      </c>
+      <c r="E16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="7">
+        <v>0.21791000000000002</v>
+      </c>
+      <c r="E17" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" s="7">
+        <v>9.3720000000000012E-2</v>
+      </c>
+      <c r="E18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="7">
+        <v>0.24805000000000002</v>
+      </c>
+      <c r="E19" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D20" s="7">
+        <v>0.25752999999999998</v>
+      </c>
+      <c r="E20" t="s">
+        <v>15</v>
+      </c>
+      <c r="F20" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D21" s="7">
+        <v>0.11076</v>
+      </c>
+      <c r="E21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D22" s="7">
+        <v>0.29315000000000002</v>
+      </c>
+      <c r="E22" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>14</v>
+      </c>
+      <c r="B23" t="s">
+        <v>112</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="D23" s="7">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="E23" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>14</v>
+      </c>
+      <c r="B24" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D24">
+        <v>2</v>
+      </c>
+      <c r="E24" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B25" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D25">
+        <v>130</v>
+      </c>
+      <c r="E25" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25" s="1"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B26" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D26">
+        <v>215</v>
+      </c>
+      <c r="F26" s="1"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B27" t="s">
+        <v>28</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D27">
+        <v>265</v>
+      </c>
+      <c r="F27" s="1"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D28">
+        <v>320</v>
+      </c>
+      <c r="F28" s="1"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>14</v>
+      </c>
+      <c r="B29" t="s">
+        <v>30</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D29">
+        <v>350</v>
+      </c>
+      <c r="F29" s="1"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>14</v>
+      </c>
+      <c r="B30" t="s">
+        <v>72</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D30">
+        <v>75</v>
+      </c>
+      <c r="F30" s="1"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>14</v>
+      </c>
+      <c r="B31" t="s">
+        <v>70</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D31">
+        <v>-75</v>
+      </c>
+      <c r="F31" s="1"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>14</v>
+      </c>
+      <c r="B32" t="s">
+        <v>71</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D32">
+        <v>-75</v>
+      </c>
+      <c r="F32" s="1"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>34</v>
+      </c>
+      <c r="B33" t="s">
+        <v>67</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D33">
+        <v>12</v>
+      </c>
+      <c r="E33" t="s">
+        <v>69</v>
+      </c>
+      <c r="F33" s="1"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>78</v>
+      </c>
+      <c r="B34" t="s">
+        <v>81</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="D34">
+        <v>0.88</v>
+      </c>
+      <c r="E34" t="s">
+        <v>78</v>
+      </c>
+      <c r="F34" s="1"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>78</v>
+      </c>
+      <c r="B35" t="s">
+        <v>82</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="D35">
+        <v>0.88</v>
+      </c>
+      <c r="E35" t="s">
+        <v>78</v>
+      </c>
+      <c r="F35" s="1"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>78</v>
+      </c>
+      <c r="B36" t="s">
+        <v>89</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="D36">
+        <v>2.25</v>
+      </c>
+      <c r="E36" t="s">
+        <v>78</v>
+      </c>
+      <c r="F36" s="1"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>78</v>
+      </c>
+      <c r="B37" t="s">
+        <v>83</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D37">
+        <v>0.61</v>
+      </c>
+      <c r="E37" t="s">
+        <v>78</v>
+      </c>
+      <c r="F37" s="1"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>78</v>
+      </c>
+      <c r="B38" t="s">
+        <v>83</v>
+      </c>
+      <c r="C38" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D38">
+        <v>0.69</v>
+      </c>
+      <c r="E38" t="s">
+        <v>78</v>
+      </c>
+      <c r="F38" s="1"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>78</v>
+      </c>
+      <c r="B39" t="s">
+        <v>84</v>
+      </c>
+      <c r="C39" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="D39">
+        <v>0.7</v>
+      </c>
+      <c r="E39" t="s">
+        <v>107</v>
+      </c>
+      <c r="F39" s="1"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>78</v>
+      </c>
+      <c r="B40" t="s">
+        <v>105</v>
+      </c>
+      <c r="C40" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="D40">
+        <v>0.9</v>
+      </c>
+      <c r="E40" t="s">
+        <v>108</v>
+      </c>
+      <c r="F40" s="1"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>78</v>
+      </c>
+      <c r="B41" t="s">
+        <v>85</v>
+      </c>
+      <c r="C41" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="D41">
+        <v>0.4</v>
+      </c>
+      <c r="E41" t="s">
+        <v>109</v>
+      </c>
+      <c r="F41" s="1"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>78</v>
+      </c>
+      <c r="B42" t="s">
+        <v>113</v>
+      </c>
+      <c r="C42" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="D42">
+        <v>4.25</v>
+      </c>
+      <c r="F42" s="1"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>78</v>
+      </c>
+      <c r="B43" t="s">
+        <v>115</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="D43">
+        <v>1.25</v>
+      </c>
+      <c r="F43" s="1"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>6</v>
+      </c>
+      <c r="B44" t="s">
+        <v>117</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D44">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>6</v>
+      </c>
+      <c r="B45" t="s">
+        <v>118</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="D45">
+        <v>2</v>
+      </c>
+      <c r="F45" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>6</v>
+      </c>
+      <c r="B46" t="s">
+        <v>117</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="D46">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>6</v>
+      </c>
+      <c r="B47" t="s">
+        <v>118</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D47">
+        <v>4</v>
+      </c>
+      <c r="F47" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>6</v>
+      </c>
+      <c r="B48" t="s">
+        <v>99</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>0.03</v>
+      </c>
+      <c r="E48" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>6</v>
+      </c>
+      <c r="B49" t="s">
+        <v>31</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D49">
+        <v>0.01</v>
+      </c>
+      <c r="E49" t="s">
+        <v>32</v>
+      </c>
+      <c r="F49" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>6</v>
+      </c>
+      <c r="B50" t="s">
+        <v>92</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D50">
+        <v>0.3</v>
+      </c>
+      <c r="E50" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>6</v>
+      </c>
+      <c r="B51" t="s">
+        <v>144</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D51">
+        <v>2030</v>
+      </c>
+      <c r="E51" t="s">
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -2027,18 +3788,1779 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEB88E62-7607-4F45-BA84-25687CEF5DCD}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="2" max="2" width="41.88671875" customWidth="1"/>
+    <col min="3" max="3" width="55" customWidth="1"/>
+    <col min="4" max="4" width="16.5546875" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" customWidth="1"/>
+    <col min="6" max="6" width="22.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2">
+        <v>2026.5</v>
+      </c>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3">
+        <v>2021</v>
+      </c>
+      <c r="F3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="D4">
+        <v>0.13500000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="D5">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6">
+        <v>0.13500000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>122</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D7">
+        <v>0.5</v>
+      </c>
+      <c r="E7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="D8">
+        <v>9.2999999999999999E-2</v>
+      </c>
+      <c r="E8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9">
+        <v>0.1</v>
+      </c>
+      <c r="E9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10">
+        <v>0.1</v>
+      </c>
+      <c r="E10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" s="7">
+        <v>0.16838500000000001</v>
+      </c>
+      <c r="E11" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" s="7">
+        <v>7.2419999999999998E-2</v>
+      </c>
+      <c r="E12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="7">
+        <v>0.19167500000000001</v>
+      </c>
+      <c r="E13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="D14">
+        <v>0.1981</v>
+      </c>
+      <c r="E14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15">
+        <v>8.5199999999999998E-2</v>
+      </c>
+      <c r="E15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D16">
+        <v>0.22550000000000001</v>
+      </c>
+      <c r="E16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="7">
+        <v>0.21791000000000002</v>
+      </c>
+      <c r="E17" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" s="7">
+        <v>9.3720000000000012E-2</v>
+      </c>
+      <c r="E18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="7">
+        <v>0.24805000000000002</v>
+      </c>
+      <c r="E19" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D20" s="7">
+        <v>0.25752999999999998</v>
+      </c>
+      <c r="E20" t="s">
+        <v>15</v>
+      </c>
+      <c r="F20" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D21" s="7">
+        <v>0.11076</v>
+      </c>
+      <c r="E21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D22" s="7">
+        <v>0.29315000000000002</v>
+      </c>
+      <c r="E22" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>14</v>
+      </c>
+      <c r="B23" t="s">
+        <v>112</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="D23" s="7">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="E23" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>14</v>
+      </c>
+      <c r="B24" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D24">
+        <v>2</v>
+      </c>
+      <c r="E24" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B25" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D25">
+        <v>130</v>
+      </c>
+      <c r="E25" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25" s="1"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B26" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D26">
+        <v>215</v>
+      </c>
+      <c r="F26" s="1"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B27" t="s">
+        <v>28</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D27">
+        <v>265</v>
+      </c>
+      <c r="F27" s="1"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D28">
+        <v>320</v>
+      </c>
+      <c r="F28" s="1"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>14</v>
+      </c>
+      <c r="B29" t="s">
+        <v>30</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D29">
+        <v>350</v>
+      </c>
+      <c r="F29" s="1"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>14</v>
+      </c>
+      <c r="B30" t="s">
+        <v>72</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D30">
+        <v>75</v>
+      </c>
+      <c r="F30" s="1"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>14</v>
+      </c>
+      <c r="B31" t="s">
+        <v>70</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D31">
+        <v>75</v>
+      </c>
+      <c r="F31" s="1"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>14</v>
+      </c>
+      <c r="B32" t="s">
+        <v>71</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D32">
+        <v>75</v>
+      </c>
+      <c r="F32" s="1"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>34</v>
+      </c>
+      <c r="B33" t="s">
+        <v>67</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D33">
+        <v>12</v>
+      </c>
+      <c r="E33" t="s">
+        <v>69</v>
+      </c>
+      <c r="F33" s="1"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>78</v>
+      </c>
+      <c r="B34" t="s">
+        <v>81</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="D34">
+        <v>0.88</v>
+      </c>
+      <c r="E34" t="s">
+        <v>78</v>
+      </c>
+      <c r="F34" s="1"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>78</v>
+      </c>
+      <c r="B35" t="s">
+        <v>82</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="D35">
+        <v>0.88</v>
+      </c>
+      <c r="E35" t="s">
+        <v>78</v>
+      </c>
+      <c r="F35" s="1"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>78</v>
+      </c>
+      <c r="B36" t="s">
+        <v>89</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="D36">
+        <v>2.25</v>
+      </c>
+      <c r="E36" t="s">
+        <v>78</v>
+      </c>
+      <c r="F36" s="1"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>78</v>
+      </c>
+      <c r="B37" t="s">
+        <v>83</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D37">
+        <v>0.61</v>
+      </c>
+      <c r="E37" t="s">
+        <v>78</v>
+      </c>
+      <c r="F37" s="1"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>78</v>
+      </c>
+      <c r="B38" t="s">
+        <v>83</v>
+      </c>
+      <c r="C38" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D38">
+        <v>0.69</v>
+      </c>
+      <c r="E38" t="s">
+        <v>78</v>
+      </c>
+      <c r="F38" s="1"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>78</v>
+      </c>
+      <c r="B39" t="s">
+        <v>84</v>
+      </c>
+      <c r="C39" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="D39">
+        <v>0.7</v>
+      </c>
+      <c r="E39" t="s">
+        <v>107</v>
+      </c>
+      <c r="F39" s="1"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>78</v>
+      </c>
+      <c r="B40" t="s">
+        <v>105</v>
+      </c>
+      <c r="C40" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="D40">
+        <v>0.9</v>
+      </c>
+      <c r="E40" t="s">
+        <v>108</v>
+      </c>
+      <c r="F40" s="1"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>78</v>
+      </c>
+      <c r="B41" t="s">
+        <v>85</v>
+      </c>
+      <c r="C41" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="D41">
+        <v>0.4</v>
+      </c>
+      <c r="E41" t="s">
+        <v>109</v>
+      </c>
+      <c r="F41" s="1"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>78</v>
+      </c>
+      <c r="B42" t="s">
+        <v>113</v>
+      </c>
+      <c r="C42" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="D42">
+        <v>4.25</v>
+      </c>
+      <c r="F42" s="1"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>78</v>
+      </c>
+      <c r="B43" t="s">
+        <v>115</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="D43">
+        <v>1.25</v>
+      </c>
+      <c r="F43" s="1"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>6</v>
+      </c>
+      <c r="B44" t="s">
+        <v>117</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D44">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>6</v>
+      </c>
+      <c r="B45" t="s">
+        <v>118</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="D45">
+        <v>2</v>
+      </c>
+      <c r="F45" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>6</v>
+      </c>
+      <c r="B46" t="s">
+        <v>117</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="D46">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>6</v>
+      </c>
+      <c r="B47" t="s">
+        <v>118</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D47">
+        <v>4</v>
+      </c>
+      <c r="F47" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>6</v>
+      </c>
+      <c r="B48" t="s">
+        <v>99</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>0.03</v>
+      </c>
+      <c r="E48" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>6</v>
+      </c>
+      <c r="B49" t="s">
+        <v>31</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D49">
+        <v>0.01</v>
+      </c>
+      <c r="E49" t="s">
+        <v>32</v>
+      </c>
+      <c r="F49" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>6</v>
+      </c>
+      <c r="B50" t="s">
+        <v>92</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D50">
+        <v>0.3</v>
+      </c>
+      <c r="E50" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>6</v>
+      </c>
+      <c r="B51" t="s">
+        <v>144</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D51">
+        <v>2030</v>
+      </c>
+      <c r="E51" t="s">
+        <v>145</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{637651EF-BBD1-4820-B575-600BCC8F4568}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="40.5546875" customWidth="1"/>
+    <col min="3" max="3" width="58.21875" customWidth="1"/>
+    <col min="4" max="4" width="14.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2">
+        <v>2026.5</v>
+      </c>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3">
+        <v>2021</v>
+      </c>
+      <c r="F3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="D4">
+        <v>0.13500000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="D5">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6">
+        <v>0.13500000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>122</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D7">
+        <v>0.5</v>
+      </c>
+      <c r="E7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="D8">
+        <v>9.2999999999999999E-2</v>
+      </c>
+      <c r="E8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9">
+        <v>0.17</v>
+      </c>
+      <c r="E9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10">
+        <v>0.37</v>
+      </c>
+      <c r="E10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" s="7">
+        <v>0.16838500000000001</v>
+      </c>
+      <c r="E11" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" s="7">
+        <v>7.2419999999999998E-2</v>
+      </c>
+      <c r="E12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="7">
+        <v>0.19167500000000001</v>
+      </c>
+      <c r="E13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="D14">
+        <v>0.1981</v>
+      </c>
+      <c r="E14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15">
+        <v>8.5199999999999998E-2</v>
+      </c>
+      <c r="E15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D16">
+        <v>0.22550000000000001</v>
+      </c>
+      <c r="E16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="7">
+        <v>0.21791000000000002</v>
+      </c>
+      <c r="E17" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" s="7">
+        <v>9.3720000000000012E-2</v>
+      </c>
+      <c r="E18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="7">
+        <v>0.24805000000000002</v>
+      </c>
+      <c r="E19" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D20" s="7">
+        <v>0.25752999999999998</v>
+      </c>
+      <c r="E20" t="s">
+        <v>15</v>
+      </c>
+      <c r="F20" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D21" s="7">
+        <v>0.11076</v>
+      </c>
+      <c r="E21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D22" s="7">
+        <v>0.29315000000000002</v>
+      </c>
+      <c r="E22" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>14</v>
+      </c>
+      <c r="B23" t="s">
+        <v>112</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="D23" s="7">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="E23" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>14</v>
+      </c>
+      <c r="B24" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D24">
+        <v>2</v>
+      </c>
+      <c r="E24" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B25" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D25">
+        <v>130</v>
+      </c>
+      <c r="E25" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25" s="1"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B26" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D26">
+        <v>215</v>
+      </c>
+      <c r="F26" s="1"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B27" t="s">
+        <v>28</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D27">
+        <v>265</v>
+      </c>
+      <c r="F27" s="1"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D28">
+        <v>320</v>
+      </c>
+      <c r="F28" s="1"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>14</v>
+      </c>
+      <c r="B29" t="s">
+        <v>30</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D29">
+        <v>350</v>
+      </c>
+      <c r="F29" s="1"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>14</v>
+      </c>
+      <c r="B30" t="s">
+        <v>72</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D30">
+        <v>75</v>
+      </c>
+      <c r="F30" s="1"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>14</v>
+      </c>
+      <c r="B31" t="s">
+        <v>70</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D31">
+        <v>75</v>
+      </c>
+      <c r="F31" s="1"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>14</v>
+      </c>
+      <c r="B32" t="s">
+        <v>71</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D32">
+        <v>75</v>
+      </c>
+      <c r="F32" s="1"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>34</v>
+      </c>
+      <c r="B33" t="s">
+        <v>67</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D33">
+        <v>12</v>
+      </c>
+      <c r="E33" t="s">
+        <v>69</v>
+      </c>
+      <c r="F33" s="1"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>78</v>
+      </c>
+      <c r="B34" t="s">
+        <v>81</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="D34">
+        <v>0.88</v>
+      </c>
+      <c r="E34" t="s">
+        <v>78</v>
+      </c>
+      <c r="F34" s="1"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>78</v>
+      </c>
+      <c r="B35" t="s">
+        <v>82</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="D35">
+        <v>0.88</v>
+      </c>
+      <c r="E35" t="s">
+        <v>78</v>
+      </c>
+      <c r="F35" s="1"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>78</v>
+      </c>
+      <c r="B36" t="s">
+        <v>89</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="D36">
+        <v>2.25</v>
+      </c>
+      <c r="E36" t="s">
+        <v>78</v>
+      </c>
+      <c r="F36" s="1"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>78</v>
+      </c>
+      <c r="B37" t="s">
+        <v>83</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D37">
+        <v>0.61</v>
+      </c>
+      <c r="E37" t="s">
+        <v>78</v>
+      </c>
+      <c r="F37" s="1"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>78</v>
+      </c>
+      <c r="B38" t="s">
+        <v>83</v>
+      </c>
+      <c r="C38" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D38">
+        <v>0.69</v>
+      </c>
+      <c r="E38" t="s">
+        <v>78</v>
+      </c>
+      <c r="F38" s="1"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>78</v>
+      </c>
+      <c r="B39" t="s">
+        <v>84</v>
+      </c>
+      <c r="C39" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="D39">
+        <v>0.7</v>
+      </c>
+      <c r="E39" t="s">
+        <v>107</v>
+      </c>
+      <c r="F39" s="1"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>78</v>
+      </c>
+      <c r="B40" t="s">
+        <v>105</v>
+      </c>
+      <c r="C40" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="D40">
+        <v>0.9</v>
+      </c>
+      <c r="E40" t="s">
+        <v>108</v>
+      </c>
+      <c r="F40" s="1"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>78</v>
+      </c>
+      <c r="B41" t="s">
+        <v>85</v>
+      </c>
+      <c r="C41" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="D41">
+        <v>0.4</v>
+      </c>
+      <c r="E41" t="s">
+        <v>109</v>
+      </c>
+      <c r="F41" s="1"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>78</v>
+      </c>
+      <c r="B42" t="s">
+        <v>113</v>
+      </c>
+      <c r="C42" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="D42">
+        <v>4.25</v>
+      </c>
+      <c r="F42" s="1"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>78</v>
+      </c>
+      <c r="B43" t="s">
+        <v>115</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="D43">
+        <v>1.25</v>
+      </c>
+      <c r="F43" s="1"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>6</v>
+      </c>
+      <c r="B44" t="s">
+        <v>117</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D44">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>6</v>
+      </c>
+      <c r="B45" t="s">
+        <v>118</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="D45">
+        <v>2</v>
+      </c>
+      <c r="F45" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>6</v>
+      </c>
+      <c r="B46" t="s">
+        <v>117</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="D46">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>6</v>
+      </c>
+      <c r="B47" t="s">
+        <v>118</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D47">
+        <v>4</v>
+      </c>
+      <c r="F47" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>6</v>
+      </c>
+      <c r="B48" t="s">
+        <v>99</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>0.03</v>
+      </c>
+      <c r="E48" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>6</v>
+      </c>
+      <c r="B49" t="s">
+        <v>31</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D49">
+        <v>0.01</v>
+      </c>
+      <c r="E49" t="s">
+        <v>32</v>
+      </c>
+      <c r="F49" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>6</v>
+      </c>
+      <c r="B50" t="s">
+        <v>92</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D50">
+        <v>0.3</v>
+      </c>
+      <c r="E50" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>6</v>
+      </c>
+      <c r="B51" t="s">
+        <v>144</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D51">
+        <v>2030</v>
+      </c>
+      <c r="E51" t="s">
+        <v>145</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated network price assumptions
</commit_message>
<xml_diff>
--- a/inst/ext_data/scenario_parameters.xlsx
+++ b/inst/ext_data/scenario_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\depmicrosimr\inst\ext_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7E7C3F1-CF76-4FA1-8E79-790198C1BDE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{480A690F-4DEA-4110-9AFD-1D9BC4B01E3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1025" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1025" uniqueCount="147">
   <si>
     <t>category</t>
   </si>
@@ -209,9 +209,6 @@
   </si>
   <si>
     <t>10% above 2026 values</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30% above </t>
   </si>
   <si>
     <t>day_network_charge_2026</t>
@@ -519,13 +516,10 @@
     <t>year time at which awareness of dynamic pricing is universal. Must be &gt; 2026.5.</t>
   </si>
   <si>
-    <t>loss averssion beta distribution alpha</t>
-  </si>
-  <si>
-    <t>loss averssion beta distribution beta</t>
-  </si>
-  <si>
     <t>EDSC</t>
+  </si>
+  <si>
+    <t>30% above 2026</t>
   </si>
 </sst>
 </file>
@@ -1017,12 +1011,12 @@
   <sheetData>
     <row r="1" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>9</v>
@@ -1036,76 +1030,76 @@
     </row>
     <row r="3" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="C3" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>102</v>
-      </c>
       <c r="D3" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="17" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>124</v>
-      </c>
       <c r="C5" s="15" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="17" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="17" t="s">
+        <v>126</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>127</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
+        <v>133</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>136</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -1183,10 +1177,10 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D4">
         <v>0.13500000000000001</v>
@@ -1197,10 +1191,10 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D5">
         <v>0.09</v>
@@ -1211,10 +1205,10 @@
         <v>12</v>
       </c>
       <c r="B6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>65</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>66</v>
       </c>
       <c r="D6">
         <v>0.13500000000000001</v>
@@ -1225,10 +1219,10 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D7">
         <v>0.5</v>
@@ -1237,7 +1231,7 @@
         <v>15</v>
       </c>
       <c r="F7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -1245,10 +1239,10 @@
         <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D8">
         <v>9.2999999999999999E-2</v>
@@ -1257,7 +1251,7 @@
         <v>15</v>
       </c>
       <c r="F8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -1265,10 +1259,10 @@
         <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D9">
         <v>0.13</v>
@@ -1277,7 +1271,7 @@
         <v>15</v>
       </c>
       <c r="F9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -1285,10 +1279,10 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D10">
         <v>0.2</v>
@@ -1360,7 +1354,7 @@
         <v>40</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D14">
         <v>0.1981</v>
@@ -1380,7 +1374,7 @@
         <v>38</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D15">
         <v>8.5199999999999998E-2</v>
@@ -1397,7 +1391,7 @@
         <v>39</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D16">
         <v>0.22550000000000001</v>
@@ -1437,10 +1431,14 @@
         <v>45</v>
       </c>
       <c r="D18" s="7">
-        <v>9.3720000000000012E-2</v>
+        <v>0.10501000000000002</v>
       </c>
       <c r="E18" t="s">
         <v>15</v>
+      </c>
+      <c r="F18" s="7">
+        <f>D17-D14</f>
+        <v>1.9810000000000022E-2</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -1454,7 +1452,7 @@
         <v>46</v>
       </c>
       <c r="D19" s="7">
-        <v>0.24805000000000002</v>
+        <v>0.24531000000000003</v>
       </c>
       <c r="E19" t="s">
         <v>15</v>
@@ -1468,7 +1466,7 @@
         <v>40</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D20" s="7">
         <v>0.25752999999999998</v>
@@ -1477,7 +1475,7 @@
         <v>15</v>
       </c>
       <c r="F20" t="s">
-        <v>50</v>
+        <v>146</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -1488,13 +1486,17 @@
         <v>38</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D21" s="7">
-        <v>0.11076</v>
+        <v>0.14462999999999998</v>
       </c>
       <c r="E21" t="s">
         <v>15</v>
+      </c>
+      <c r="F21" s="7">
+        <f>(D20-D14)</f>
+        <v>5.9429999999999983E-2</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -1505,30 +1507,31 @@
         <v>39</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D22" s="7">
-        <v>0.29315000000000002</v>
+        <v>0.28493000000000002</v>
       </c>
       <c r="E22" t="s">
         <v>15</v>
       </c>
+      <c r="F22" s="7"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>14</v>
       </c>
       <c r="B23" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D23" s="7">
         <v>0.33333333333333331</v>
       </c>
       <c r="E23" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -1634,10 +1637,10 @@
         <v>14</v>
       </c>
       <c r="B30" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D30">
         <v>75</v>
@@ -1649,10 +1652,10 @@
         <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D31">
         <v>75</v>
@@ -1664,10 +1667,10 @@
         <v>14</v>
       </c>
       <c r="B32" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D32">
         <v>75</v>
@@ -1679,172 +1682,172 @@
         <v>34</v>
       </c>
       <c r="B33" t="s">
+        <v>66</v>
+      </c>
+      <c r="C33" s="6" t="s">
         <v>67</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>68</v>
       </c>
       <c r="D33">
         <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F33" s="1"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>77</v>
+      </c>
+      <c r="B34" t="s">
+        <v>80</v>
+      </c>
+      <c r="C34" s="13" t="s">
         <v>78</v>
-      </c>
-      <c r="B34" t="s">
-        <v>81</v>
-      </c>
-      <c r="C34" s="13" t="s">
-        <v>79</v>
       </c>
       <c r="D34">
         <v>0.88</v>
       </c>
       <c r="E34" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F34" s="1"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B35" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D35">
         <v>0.88</v>
       </c>
       <c r="E35" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F35" s="1"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B36" t="s">
+        <v>88</v>
+      </c>
+      <c r="C36" s="13" t="s">
         <v>89</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>90</v>
       </c>
       <c r="D36">
         <v>2.25</v>
       </c>
       <c r="E36" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F36" s="1"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B37" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D37">
         <v>0.61</v>
       </c>
       <c r="E37" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F37" s="1"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B38" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D38">
         <v>0.69</v>
       </c>
       <c r="E38" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F38" s="1"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B39" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D39">
         <v>0.7</v>
       </c>
       <c r="E39" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F39" s="1"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B40" t="s">
+        <v>104</v>
+      </c>
+      <c r="C40" s="13" t="s">
         <v>105</v>
-      </c>
-      <c r="C40" s="13" t="s">
-        <v>106</v>
       </c>
       <c r="D40">
         <v>0.9</v>
       </c>
       <c r="E40" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F40" s="1"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B41" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D41">
         <v>0.4</v>
       </c>
       <c r="E41" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F41" s="1"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B42" t="s">
+        <v>112</v>
+      </c>
+      <c r="C42" s="13" t="s">
         <v>113</v>
-      </c>
-      <c r="C42" s="13" t="s">
-        <v>114</v>
       </c>
       <c r="D42">
         <v>4.25</v>
@@ -1853,13 +1856,13 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B43" t="s">
+        <v>114</v>
+      </c>
+      <c r="C43" s="13" t="s">
         <v>115</v>
-      </c>
-      <c r="C43" s="13" t="s">
-        <v>116</v>
       </c>
       <c r="D43">
         <v>1.25</v>
@@ -1871,10 +1874,10 @@
         <v>6</v>
       </c>
       <c r="B44" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D44">
         <v>2</v>
@@ -1885,16 +1888,16 @@
         <v>6</v>
       </c>
       <c r="B45" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D45">
         <v>2</v>
       </c>
       <c r="F45" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -1902,10 +1905,10 @@
         <v>6</v>
       </c>
       <c r="B46" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D46">
         <v>2</v>
@@ -1916,16 +1919,16 @@
         <v>6</v>
       </c>
       <c r="B47" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D47">
         <v>4</v>
       </c>
       <c r="F47" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -1933,7 +1936,7 @@
         <v>6</v>
       </c>
       <c r="B48" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>7</v>
@@ -1942,7 +1945,7 @@
         <v>0.03</v>
       </c>
       <c r="E48" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -1962,7 +1965,7 @@
         <v>32</v>
       </c>
       <c r="F49" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -1970,16 +1973,16 @@
         <v>6</v>
       </c>
       <c r="B50" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D50">
         <v>0.3</v>
       </c>
       <c r="E50" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
@@ -1987,16 +1990,16 @@
         <v>6</v>
       </c>
       <c r="B51" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D51">
         <v>2030</v>
       </c>
       <c r="E51" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -2074,10 +2077,10 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D4">
         <v>0.13500000000000001</v>
@@ -2088,10 +2091,10 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D5">
         <v>0.09</v>
@@ -2102,10 +2105,10 @@
         <v>12</v>
       </c>
       <c r="B6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>65</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>66</v>
       </c>
       <c r="D6">
         <v>0.13500000000000001</v>
@@ -2116,10 +2119,10 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D7">
         <v>0.5</v>
@@ -2128,7 +2131,7 @@
         <v>15</v>
       </c>
       <c r="F7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -2136,10 +2139,10 @@
         <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D8">
         <v>9.2999999999999999E-2</v>
@@ -2148,7 +2151,7 @@
         <v>15</v>
       </c>
       <c r="F8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -2156,10 +2159,10 @@
         <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D9">
         <v>0.13</v>
@@ -2168,7 +2171,7 @@
         <v>15</v>
       </c>
       <c r="F9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -2176,10 +2179,10 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D10">
         <v>0.2</v>
@@ -2251,7 +2254,7 @@
         <v>40</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D14">
         <v>0.1981</v>
@@ -2271,7 +2274,7 @@
         <v>38</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D15">
         <v>8.5199999999999998E-2</v>
@@ -2288,7 +2291,7 @@
         <v>39</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D16">
         <v>0.22550000000000001</v>
@@ -2328,10 +2331,14 @@
         <v>45</v>
       </c>
       <c r="D18" s="7">
-        <v>9.3720000000000012E-2</v>
+        <v>0.10501000000000002</v>
       </c>
       <c r="E18" t="s">
         <v>15</v>
+      </c>
+      <c r="F18" s="7">
+        <f>D17-D14</f>
+        <v>1.9810000000000022E-2</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -2345,7 +2352,7 @@
         <v>46</v>
       </c>
       <c r="D19" s="7">
-        <v>0.24805000000000002</v>
+        <v>0.24531000000000003</v>
       </c>
       <c r="E19" t="s">
         <v>15</v>
@@ -2359,7 +2366,7 @@
         <v>40</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D20" s="7">
         <v>0.25752999999999998</v>
@@ -2368,7 +2375,7 @@
         <v>15</v>
       </c>
       <c r="F20" t="s">
-        <v>50</v>
+        <v>146</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -2379,13 +2386,17 @@
         <v>38</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D21" s="7">
-        <v>0.11076</v>
+        <v>0.14462999999999998</v>
       </c>
       <c r="E21" t="s">
         <v>15</v>
+      </c>
+      <c r="F21" s="7">
+        <f>(D20-D14)</f>
+        <v>5.9429999999999983E-2</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -2396,30 +2407,31 @@
         <v>39</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D22" s="7">
-        <v>0.29315000000000002</v>
+        <v>0.28493000000000002</v>
       </c>
       <c r="E22" t="s">
         <v>15</v>
       </c>
+      <c r="F22" s="7"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>14</v>
       </c>
       <c r="B23" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D23" s="7">
         <v>0.33333333333333331</v>
       </c>
       <c r="E23" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -2525,10 +2537,10 @@
         <v>14</v>
       </c>
       <c r="B30" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D30">
         <v>75</v>
@@ -2540,10 +2552,10 @@
         <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D31">
         <v>0</v>
@@ -2555,10 +2567,10 @@
         <v>14</v>
       </c>
       <c r="B32" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D32">
         <v>0</v>
@@ -2570,172 +2582,172 @@
         <v>34</v>
       </c>
       <c r="B33" t="s">
+        <v>66</v>
+      </c>
+      <c r="C33" s="6" t="s">
         <v>67</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>68</v>
       </c>
       <c r="D33">
         <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F33" s="1"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>77</v>
+      </c>
+      <c r="B34" t="s">
+        <v>80</v>
+      </c>
+      <c r="C34" s="13" t="s">
         <v>78</v>
-      </c>
-      <c r="B34" t="s">
-        <v>81</v>
-      </c>
-      <c r="C34" s="13" t="s">
-        <v>79</v>
       </c>
       <c r="D34">
         <v>0.88</v>
       </c>
       <c r="E34" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F34" s="1"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B35" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D35">
         <v>0.88</v>
       </c>
       <c r="E35" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F35" s="1"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B36" t="s">
+        <v>88</v>
+      </c>
+      <c r="C36" s="13" t="s">
         <v>89</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>90</v>
       </c>
       <c r="D36">
         <v>2.25</v>
       </c>
       <c r="E36" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F36" s="1"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B37" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D37">
         <v>0.61</v>
       </c>
       <c r="E37" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F37" s="1"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B38" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D38">
         <v>0.69</v>
       </c>
       <c r="E38" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F38" s="1"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B39" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D39">
         <v>0.7</v>
       </c>
       <c r="E39" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F39" s="1"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B40" t="s">
+        <v>104</v>
+      </c>
+      <c r="C40" s="13" t="s">
         <v>105</v>
-      </c>
-      <c r="C40" s="13" t="s">
-        <v>106</v>
       </c>
       <c r="D40">
         <v>0.9</v>
       </c>
       <c r="E40" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F40" s="1"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B41" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D41">
         <v>0.4</v>
       </c>
       <c r="E41" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F41" s="1"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B42" t="s">
+        <v>112</v>
+      </c>
+      <c r="C42" s="13" t="s">
         <v>113</v>
-      </c>
-      <c r="C42" s="13" t="s">
-        <v>114</v>
       </c>
       <c r="D42">
         <v>4.25</v>
@@ -2744,13 +2756,13 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B43" t="s">
+        <v>114</v>
+      </c>
+      <c r="C43" s="13" t="s">
         <v>115</v>
-      </c>
-      <c r="C43" s="13" t="s">
-        <v>116</v>
       </c>
       <c r="D43">
         <v>1.25</v>
@@ -2762,10 +2774,10 @@
         <v>6</v>
       </c>
       <c r="B44" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D44">
         <v>2</v>
@@ -2776,16 +2788,16 @@
         <v>6</v>
       </c>
       <c r="B45" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D45">
         <v>2</v>
       </c>
       <c r="F45" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -2793,10 +2805,10 @@
         <v>6</v>
       </c>
       <c r="B46" t="s">
-        <v>146</v>
+        <v>116</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D46">
         <v>2</v>
@@ -2807,16 +2819,16 @@
         <v>6</v>
       </c>
       <c r="B47" t="s">
-        <v>147</v>
+        <v>117</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D47">
         <v>4</v>
       </c>
       <c r="F47" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -2824,7 +2836,7 @@
         <v>6</v>
       </c>
       <c r="B48" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>7</v>
@@ -2833,7 +2845,7 @@
         <v>0.03</v>
       </c>
       <c r="E48" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -2853,7 +2865,7 @@
         <v>32</v>
       </c>
       <c r="F49" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -2861,16 +2873,16 @@
         <v>6</v>
       </c>
       <c r="B50" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D50">
         <v>0.3</v>
       </c>
       <c r="E50" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
@@ -2878,16 +2890,16 @@
         <v>6</v>
       </c>
       <c r="B51" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D51">
         <v>2030</v>
       </c>
       <c r="E51" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -2965,10 +2977,10 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D4">
         <v>0.13500000000000001</v>
@@ -2979,10 +2991,10 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D5">
         <v>0.09</v>
@@ -2993,10 +3005,10 @@
         <v>12</v>
       </c>
       <c r="B6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>65</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>66</v>
       </c>
       <c r="D6">
         <v>0.13500000000000001</v>
@@ -3007,10 +3019,10 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D7">
         <v>0.5</v>
@@ -3019,7 +3031,7 @@
         <v>15</v>
       </c>
       <c r="F7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -3027,10 +3039,10 @@
         <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D8">
         <v>9.2999999999999999E-2</v>
@@ -3039,7 +3051,7 @@
         <v>15</v>
       </c>
       <c r="F8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -3047,10 +3059,10 @@
         <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D9">
         <v>0.13</v>
@@ -3059,7 +3071,7 @@
         <v>15</v>
       </c>
       <c r="F9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -3067,10 +3079,10 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D10">
         <v>0.2</v>
@@ -3142,7 +3154,7 @@
         <v>40</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D14">
         <v>0.1981</v>
@@ -3162,7 +3174,7 @@
         <v>38</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D15">
         <v>8.5199999999999998E-2</v>
@@ -3179,7 +3191,7 @@
         <v>39</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D16">
         <v>0.22550000000000001</v>
@@ -3219,10 +3231,14 @@
         <v>45</v>
       </c>
       <c r="D18" s="7">
-        <v>9.3720000000000012E-2</v>
+        <v>0.10501000000000002</v>
       </c>
       <c r="E18" t="s">
         <v>15</v>
+      </c>
+      <c r="F18" s="7">
+        <f>D17-D14</f>
+        <v>1.9810000000000022E-2</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -3236,7 +3252,7 @@
         <v>46</v>
       </c>
       <c r="D19" s="7">
-        <v>0.24805000000000002</v>
+        <v>0.24531000000000003</v>
       </c>
       <c r="E19" t="s">
         <v>15</v>
@@ -3250,7 +3266,7 @@
         <v>40</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D20" s="7">
         <v>0.25752999999999998</v>
@@ -3259,7 +3275,7 @@
         <v>15</v>
       </c>
       <c r="F20" t="s">
-        <v>50</v>
+        <v>146</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -3270,13 +3286,17 @@
         <v>38</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D21" s="7">
-        <v>0.11076</v>
+        <v>0.14462999999999998</v>
       </c>
       <c r="E21" t="s">
         <v>15</v>
+      </c>
+      <c r="F21" s="7">
+        <f>(D20-D14)</f>
+        <v>5.9429999999999983E-2</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -3287,30 +3307,31 @@
         <v>39</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D22" s="7">
-        <v>0.29315000000000002</v>
+        <v>0.28493000000000002</v>
       </c>
       <c r="E22" t="s">
         <v>15</v>
       </c>
+      <c r="F22" s="7"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>14</v>
       </c>
       <c r="B23" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D23" s="7">
         <v>0.33333333333333331</v>
       </c>
       <c r="E23" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -3416,10 +3437,10 @@
         <v>14</v>
       </c>
       <c r="B30" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D30">
         <v>75</v>
@@ -3431,10 +3452,10 @@
         <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D31">
         <v>-75</v>
@@ -3446,10 +3467,10 @@
         <v>14</v>
       </c>
       <c r="B32" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D32">
         <v>-75</v>
@@ -3461,172 +3482,172 @@
         <v>34</v>
       </c>
       <c r="B33" t="s">
+        <v>66</v>
+      </c>
+      <c r="C33" s="6" t="s">
         <v>67</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>68</v>
       </c>
       <c r="D33">
         <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F33" s="1"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>77</v>
+      </c>
+      <c r="B34" t="s">
+        <v>80</v>
+      </c>
+      <c r="C34" s="13" t="s">
         <v>78</v>
-      </c>
-      <c r="B34" t="s">
-        <v>81</v>
-      </c>
-      <c r="C34" s="13" t="s">
-        <v>79</v>
       </c>
       <c r="D34">
         <v>0.88</v>
       </c>
       <c r="E34" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F34" s="1"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B35" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D35">
         <v>0.88</v>
       </c>
       <c r="E35" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F35" s="1"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B36" t="s">
+        <v>88</v>
+      </c>
+      <c r="C36" s="13" t="s">
         <v>89</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>90</v>
       </c>
       <c r="D36">
         <v>2.25</v>
       </c>
       <c r="E36" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F36" s="1"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B37" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D37">
         <v>0.61</v>
       </c>
       <c r="E37" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F37" s="1"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B38" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D38">
         <v>0.69</v>
       </c>
       <c r="E38" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F38" s="1"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B39" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D39">
         <v>0.7</v>
       </c>
       <c r="E39" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F39" s="1"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B40" t="s">
+        <v>104</v>
+      </c>
+      <c r="C40" s="13" t="s">
         <v>105</v>
-      </c>
-      <c r="C40" s="13" t="s">
-        <v>106</v>
       </c>
       <c r="D40">
         <v>0.9</v>
       </c>
       <c r="E40" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F40" s="1"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B41" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D41">
         <v>0.4</v>
       </c>
       <c r="E41" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F41" s="1"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B42" t="s">
+        <v>112</v>
+      </c>
+      <c r="C42" s="13" t="s">
         <v>113</v>
-      </c>
-      <c r="C42" s="13" t="s">
-        <v>114</v>
       </c>
       <c r="D42">
         <v>4.25</v>
@@ -3635,13 +3656,13 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B43" t="s">
+        <v>114</v>
+      </c>
+      <c r="C43" s="13" t="s">
         <v>115</v>
-      </c>
-      <c r="C43" s="13" t="s">
-        <v>116</v>
       </c>
       <c r="D43">
         <v>1.25</v>
@@ -3653,10 +3674,10 @@
         <v>6</v>
       </c>
       <c r="B44" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D44">
         <v>2</v>
@@ -3667,16 +3688,16 @@
         <v>6</v>
       </c>
       <c r="B45" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D45">
         <v>2</v>
       </c>
       <c r="F45" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -3684,10 +3705,10 @@
         <v>6</v>
       </c>
       <c r="B46" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D46">
         <v>2</v>
@@ -3698,16 +3719,16 @@
         <v>6</v>
       </c>
       <c r="B47" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D47">
         <v>4</v>
       </c>
       <c r="F47" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -3715,7 +3736,7 @@
         <v>6</v>
       </c>
       <c r="B48" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>7</v>
@@ -3724,7 +3745,7 @@
         <v>0.03</v>
       </c>
       <c r="E48" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -3744,7 +3765,7 @@
         <v>32</v>
       </c>
       <c r="F49" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -3752,16 +3773,16 @@
         <v>6</v>
       </c>
       <c r="B50" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D50">
         <v>0.3</v>
       </c>
       <c r="E50" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
@@ -3769,16 +3790,16 @@
         <v>6</v>
       </c>
       <c r="B51" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D51">
         <v>2030</v>
       </c>
       <c r="E51" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -3856,10 +3877,10 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D4">
         <v>0.13500000000000001</v>
@@ -3870,10 +3891,10 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D5">
         <v>0.09</v>
@@ -3884,10 +3905,10 @@
         <v>12</v>
       </c>
       <c r="B6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>65</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>66</v>
       </c>
       <c r="D6">
         <v>0.13500000000000001</v>
@@ -3898,10 +3919,10 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D7">
         <v>0.5</v>
@@ -3910,7 +3931,7 @@
         <v>15</v>
       </c>
       <c r="F7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -3918,10 +3939,10 @@
         <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D8">
         <v>9.2999999999999999E-2</v>
@@ -3930,7 +3951,7 @@
         <v>15</v>
       </c>
       <c r="F8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -3938,10 +3959,10 @@
         <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D9">
         <v>0.1</v>
@@ -3950,7 +3971,7 @@
         <v>15</v>
       </c>
       <c r="F9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -3958,10 +3979,10 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D10">
         <v>0.1</v>
@@ -4033,7 +4054,7 @@
         <v>40</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D14">
         <v>0.1981</v>
@@ -4053,7 +4074,7 @@
         <v>38</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D15">
         <v>8.5199999999999998E-2</v>
@@ -4070,7 +4091,7 @@
         <v>39</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D16">
         <v>0.22550000000000001</v>
@@ -4110,10 +4131,14 @@
         <v>45</v>
       </c>
       <c r="D18" s="7">
-        <v>9.3720000000000012E-2</v>
+        <v>0.10501000000000002</v>
       </c>
       <c r="E18" t="s">
         <v>15</v>
+      </c>
+      <c r="F18" s="7">
+        <f>D17-D14</f>
+        <v>1.9810000000000022E-2</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -4127,7 +4152,7 @@
         <v>46</v>
       </c>
       <c r="D19" s="7">
-        <v>0.24805000000000002</v>
+        <v>0.24531000000000003</v>
       </c>
       <c r="E19" t="s">
         <v>15</v>
@@ -4141,7 +4166,7 @@
         <v>40</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D20" s="7">
         <v>0.25752999999999998</v>
@@ -4150,7 +4175,7 @@
         <v>15</v>
       </c>
       <c r="F20" t="s">
-        <v>50</v>
+        <v>146</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -4161,13 +4186,17 @@
         <v>38</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D21" s="7">
-        <v>0.11076</v>
+        <v>0.14462999999999998</v>
       </c>
       <c r="E21" t="s">
         <v>15</v>
+      </c>
+      <c r="F21" s="7">
+        <f>(D20-D14)</f>
+        <v>5.9429999999999983E-2</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -4178,30 +4207,31 @@
         <v>39</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D22" s="7">
-        <v>0.29315000000000002</v>
+        <v>0.28493000000000002</v>
       </c>
       <c r="E22" t="s">
         <v>15</v>
       </c>
+      <c r="F22" s="7"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>14</v>
       </c>
       <c r="B23" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D23" s="7">
         <v>0.33333333333333331</v>
       </c>
       <c r="E23" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -4307,10 +4337,10 @@
         <v>14</v>
       </c>
       <c r="B30" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D30">
         <v>75</v>
@@ -4322,10 +4352,10 @@
         <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D31">
         <v>75</v>
@@ -4337,10 +4367,10 @@
         <v>14</v>
       </c>
       <c r="B32" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D32">
         <v>75</v>
@@ -4352,172 +4382,172 @@
         <v>34</v>
       </c>
       <c r="B33" t="s">
+        <v>66</v>
+      </c>
+      <c r="C33" s="6" t="s">
         <v>67</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>68</v>
       </c>
       <c r="D33">
         <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F33" s="1"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>77</v>
+      </c>
+      <c r="B34" t="s">
+        <v>80</v>
+      </c>
+      <c r="C34" s="13" t="s">
         <v>78</v>
-      </c>
-      <c r="B34" t="s">
-        <v>81</v>
-      </c>
-      <c r="C34" s="13" t="s">
-        <v>79</v>
       </c>
       <c r="D34">
         <v>0.88</v>
       </c>
       <c r="E34" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F34" s="1"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B35" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D35">
         <v>0.88</v>
       </c>
       <c r="E35" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F35" s="1"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B36" t="s">
+        <v>88</v>
+      </c>
+      <c r="C36" s="13" t="s">
         <v>89</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>90</v>
       </c>
       <c r="D36">
         <v>2.25</v>
       </c>
       <c r="E36" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F36" s="1"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B37" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D37">
         <v>0.61</v>
       </c>
       <c r="E37" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F37" s="1"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B38" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D38">
         <v>0.69</v>
       </c>
       <c r="E38" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F38" s="1"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B39" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D39">
         <v>0.7</v>
       </c>
       <c r="E39" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F39" s="1"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B40" t="s">
+        <v>104</v>
+      </c>
+      <c r="C40" s="13" t="s">
         <v>105</v>
-      </c>
-      <c r="C40" s="13" t="s">
-        <v>106</v>
       </c>
       <c r="D40">
         <v>0.9</v>
       </c>
       <c r="E40" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F40" s="1"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B41" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D41">
         <v>0.4</v>
       </c>
       <c r="E41" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F41" s="1"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B42" t="s">
+        <v>112</v>
+      </c>
+      <c r="C42" s="13" t="s">
         <v>113</v>
-      </c>
-      <c r="C42" s="13" t="s">
-        <v>114</v>
       </c>
       <c r="D42">
         <v>4.25</v>
@@ -4526,13 +4556,13 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B43" t="s">
+        <v>114</v>
+      </c>
+      <c r="C43" s="13" t="s">
         <v>115</v>
-      </c>
-      <c r="C43" s="13" t="s">
-        <v>116</v>
       </c>
       <c r="D43">
         <v>1.25</v>
@@ -4544,10 +4574,10 @@
         <v>6</v>
       </c>
       <c r="B44" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D44">
         <v>2</v>
@@ -4558,16 +4588,16 @@
         <v>6</v>
       </c>
       <c r="B45" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D45">
         <v>2</v>
       </c>
       <c r="F45" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -4575,10 +4605,10 @@
         <v>6</v>
       </c>
       <c r="B46" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D46">
         <v>2</v>
@@ -4589,16 +4619,16 @@
         <v>6</v>
       </c>
       <c r="B47" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D47">
         <v>4</v>
       </c>
       <c r="F47" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -4606,7 +4636,7 @@
         <v>6</v>
       </c>
       <c r="B48" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>7</v>
@@ -4615,7 +4645,7 @@
         <v>0.03</v>
       </c>
       <c r="E48" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -4635,7 +4665,7 @@
         <v>32</v>
       </c>
       <c r="F49" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -4643,16 +4673,16 @@
         <v>6</v>
       </c>
       <c r="B50" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D50">
         <v>0.3</v>
       </c>
       <c r="E50" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
@@ -4660,16 +4690,16 @@
         <v>6</v>
       </c>
       <c r="B51" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D51">
         <v>2030</v>
       </c>
       <c r="E51" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -4744,10 +4774,10 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D4">
         <v>0.13500000000000001</v>
@@ -4758,10 +4788,10 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D5">
         <v>0.09</v>
@@ -4772,10 +4802,10 @@
         <v>12</v>
       </c>
       <c r="B6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>65</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>66</v>
       </c>
       <c r="D6">
         <v>0.13500000000000001</v>
@@ -4786,10 +4816,10 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D7">
         <v>0.5</v>
@@ -4798,7 +4828,7 @@
         <v>15</v>
       </c>
       <c r="F7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -4806,10 +4836,10 @@
         <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D8">
         <v>9.2999999999999999E-2</v>
@@ -4818,7 +4848,7 @@
         <v>15</v>
       </c>
       <c r="F8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -4826,19 +4856,19 @@
         <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D9">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="E9" t="s">
         <v>15</v>
       </c>
       <c r="F9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -4846,13 +4876,13 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D10">
-        <v>0.37</v>
+        <v>0.4</v>
       </c>
       <c r="E10" t="s">
         <v>15</v>
@@ -4921,7 +4951,7 @@
         <v>40</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D14">
         <v>0.1981</v>
@@ -4941,7 +4971,7 @@
         <v>38</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D15">
         <v>8.5199999999999998E-2</v>
@@ -4958,7 +4988,7 @@
         <v>39</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D16">
         <v>0.22550000000000001</v>
@@ -4998,10 +5028,14 @@
         <v>45</v>
       </c>
       <c r="D18" s="7">
-        <v>9.3720000000000012E-2</v>
+        <v>0.10501000000000002</v>
       </c>
       <c r="E18" t="s">
         <v>15</v>
+      </c>
+      <c r="F18" s="7">
+        <f>D17-D14</f>
+        <v>1.9810000000000022E-2</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -5015,7 +5049,7 @@
         <v>46</v>
       </c>
       <c r="D19" s="7">
-        <v>0.24805000000000002</v>
+        <v>0.24531000000000003</v>
       </c>
       <c r="E19" t="s">
         <v>15</v>
@@ -5029,7 +5063,7 @@
         <v>40</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D20" s="7">
         <v>0.25752999999999998</v>
@@ -5038,7 +5072,7 @@
         <v>15</v>
       </c>
       <c r="F20" t="s">
-        <v>50</v>
+        <v>146</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -5049,13 +5083,17 @@
         <v>38</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D21" s="7">
-        <v>0.11076</v>
+        <v>0.14462999999999998</v>
       </c>
       <c r="E21" t="s">
         <v>15</v>
+      </c>
+      <c r="F21" s="7">
+        <f>(D20-D14)</f>
+        <v>5.9429999999999983E-2</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -5066,30 +5104,31 @@
         <v>39</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D22" s="7">
-        <v>0.29315000000000002</v>
+        <v>0.28493000000000002</v>
       </c>
       <c r="E22" t="s">
         <v>15</v>
       </c>
+      <c r="F22" s="7"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>14</v>
       </c>
       <c r="B23" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D23" s="7">
         <v>0.33333333333333331</v>
       </c>
       <c r="E23" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -5195,10 +5234,10 @@
         <v>14</v>
       </c>
       <c r="B30" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D30">
         <v>75</v>
@@ -5210,10 +5249,10 @@
         <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D31">
         <v>75</v>
@@ -5225,10 +5264,10 @@
         <v>14</v>
       </c>
       <c r="B32" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D32">
         <v>75</v>
@@ -5240,172 +5279,172 @@
         <v>34</v>
       </c>
       <c r="B33" t="s">
+        <v>66</v>
+      </c>
+      <c r="C33" s="6" t="s">
         <v>67</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>68</v>
       </c>
       <c r="D33">
         <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F33" s="1"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>77</v>
+      </c>
+      <c r="B34" t="s">
+        <v>80</v>
+      </c>
+      <c r="C34" s="13" t="s">
         <v>78</v>
-      </c>
-      <c r="B34" t="s">
-        <v>81</v>
-      </c>
-      <c r="C34" s="13" t="s">
-        <v>79</v>
       </c>
       <c r="D34">
         <v>0.88</v>
       </c>
       <c r="E34" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F34" s="1"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B35" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D35">
         <v>0.88</v>
       </c>
       <c r="E35" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F35" s="1"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B36" t="s">
+        <v>88</v>
+      </c>
+      <c r="C36" s="13" t="s">
         <v>89</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>90</v>
       </c>
       <c r="D36">
         <v>2.25</v>
       </c>
       <c r="E36" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F36" s="1"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B37" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D37">
         <v>0.61</v>
       </c>
       <c r="E37" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F37" s="1"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B38" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D38">
         <v>0.69</v>
       </c>
       <c r="E38" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F38" s="1"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B39" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D39">
         <v>0.7</v>
       </c>
       <c r="E39" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F39" s="1"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B40" t="s">
+        <v>104</v>
+      </c>
+      <c r="C40" s="13" t="s">
         <v>105</v>
-      </c>
-      <c r="C40" s="13" t="s">
-        <v>106</v>
       </c>
       <c r="D40">
         <v>0.9</v>
       </c>
       <c r="E40" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F40" s="1"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B41" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D41">
         <v>0.4</v>
       </c>
       <c r="E41" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F41" s="1"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B42" t="s">
+        <v>112</v>
+      </c>
+      <c r="C42" s="13" t="s">
         <v>113</v>
-      </c>
-      <c r="C42" s="13" t="s">
-        <v>114</v>
       </c>
       <c r="D42">
         <v>4.25</v>
@@ -5414,13 +5453,13 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B43" t="s">
+        <v>114</v>
+      </c>
+      <c r="C43" s="13" t="s">
         <v>115</v>
-      </c>
-      <c r="C43" s="13" t="s">
-        <v>116</v>
       </c>
       <c r="D43">
         <v>1.25</v>
@@ -5432,10 +5471,10 @@
         <v>6</v>
       </c>
       <c r="B44" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D44">
         <v>2</v>
@@ -5446,16 +5485,16 @@
         <v>6</v>
       </c>
       <c r="B45" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D45">
         <v>2</v>
       </c>
       <c r="F45" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -5463,10 +5502,10 @@
         <v>6</v>
       </c>
       <c r="B46" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D46">
         <v>2</v>
@@ -5477,16 +5516,16 @@
         <v>6</v>
       </c>
       <c r="B47" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D47">
         <v>4</v>
       </c>
       <c r="F47" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -5494,7 +5533,7 @@
         <v>6</v>
       </c>
       <c r="B48" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>7</v>
@@ -5503,7 +5542,7 @@
         <v>0.03</v>
       </c>
       <c r="E48" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -5523,7 +5562,7 @@
         <v>32</v>
       </c>
       <c r="F49" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -5531,16 +5570,16 @@
         <v>6</v>
       </c>
       <c r="B50" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D50">
         <v>0.3</v>
       </c>
       <c r="E50" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
@@ -5548,16 +5587,16 @@
         <v>6</v>
       </c>
       <c r="B51" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D51">
         <v>2030</v>
       </c>
       <c r="E51" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
price simulation extended to 2045
</commit_message>
<xml_diff>
--- a/inst/ext_data/scenario_parameters.xlsx
+++ b/inst/ext_data/scenario_parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\depmicrosimr\inst\ext_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF6C5305-10D7-4F4A-B652-5CA6E2557E01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6A03693-F782-448A-80CF-585175EB55AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Description" sheetId="7" r:id="rId1"/>
@@ -1942,7 +1942,7 @@
         <v>7</v>
       </c>
       <c r="D48">
-        <v>2.7E-2</v>
+        <v>0.03</v>
       </c>
       <c r="E48" t="s">
         <v>102</v>
@@ -1979,7 +1979,7 @@
         <v>139</v>
       </c>
       <c r="D50">
-        <v>0.33</v>
+        <v>2.7E-2</v>
       </c>
       <c r="E50" t="s">
         <v>140</v>
@@ -1996,7 +1996,7 @@
         <v>142</v>
       </c>
       <c r="D51">
-        <v>2030</v>
+        <v>2028.5</v>
       </c>
       <c r="E51" t="s">
         <v>144</v>
@@ -2714,7 +2714,7 @@
         <v>105</v>
       </c>
       <c r="D40">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="E40" t="s">
         <v>107</v>
@@ -2732,7 +2732,7 @@
         <v>87</v>
       </c>
       <c r="D41">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="E41" t="s">
         <v>108</v>
@@ -2842,7 +2842,7 @@
         <v>7</v>
       </c>
       <c r="D48">
-        <v>0.03</v>
+        <v>2.7E-2</v>
       </c>
       <c r="E48" t="s">
         <v>102</v>
@@ -2879,7 +2879,7 @@
         <v>139</v>
       </c>
       <c r="D50">
-        <v>0.3</v>
+        <v>0.33</v>
       </c>
       <c r="E50" t="s">
         <v>140</v>
@@ -2896,7 +2896,7 @@
         <v>142</v>
       </c>
       <c r="D51">
-        <v>2030</v>
+        <v>2028.5</v>
       </c>
       <c r="E51" t="s">
         <v>144</v>
@@ -3614,7 +3614,7 @@
         <v>105</v>
       </c>
       <c r="D40">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="E40" t="s">
         <v>107</v>
@@ -3632,7 +3632,7 @@
         <v>87</v>
       </c>
       <c r="D41">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="E41" t="s">
         <v>108</v>
@@ -3742,7 +3742,7 @@
         <v>7</v>
       </c>
       <c r="D48">
-        <v>0.03</v>
+        <v>2.7E-2</v>
       </c>
       <c r="E48" t="s">
         <v>102</v>
@@ -3779,7 +3779,7 @@
         <v>139</v>
       </c>
       <c r="D50">
-        <v>0.3</v>
+        <v>0.33</v>
       </c>
       <c r="E50" t="s">
         <v>140</v>
@@ -3796,7 +3796,7 @@
         <v>142</v>
       </c>
       <c r="D51">
-        <v>2030</v>
+        <v>2028.5</v>
       </c>
       <c r="E51" t="s">
         <v>144</v>
@@ -4358,7 +4358,7 @@
         <v>96</v>
       </c>
       <c r="D31">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="F31" s="1"/>
     </row>
@@ -4373,7 +4373,7 @@
         <v>97</v>
       </c>
       <c r="D32">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="F32" s="1"/>
     </row>
@@ -4514,7 +4514,7 @@
         <v>105</v>
       </c>
       <c r="D40">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="E40" t="s">
         <v>107</v>
@@ -4532,7 +4532,7 @@
         <v>87</v>
       </c>
       <c r="D41">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="E41" t="s">
         <v>108</v>
@@ -4642,7 +4642,7 @@
         <v>7</v>
       </c>
       <c r="D48">
-        <v>0.03</v>
+        <v>2.7E-2</v>
       </c>
       <c r="E48" t="s">
         <v>102</v>
@@ -4679,7 +4679,7 @@
         <v>139</v>
       </c>
       <c r="D50">
-        <v>0.3</v>
+        <v>0.33</v>
       </c>
       <c r="E50" t="s">
         <v>140</v>
@@ -4696,7 +4696,7 @@
         <v>142</v>
       </c>
       <c r="D51">
-        <v>2030</v>
+        <v>2028.5</v>
       </c>
       <c r="E51" t="s">
         <v>144</v>
@@ -4862,7 +4862,7 @@
         <v>58</v>
       </c>
       <c r="D9">
-        <v>0.15</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="E9" t="s">
         <v>15</v>
@@ -4882,7 +4882,7 @@
         <v>59</v>
       </c>
       <c r="D10">
-        <v>0.4</v>
+        <v>0.37</v>
       </c>
       <c r="E10" t="s">
         <v>15</v>
@@ -5255,7 +5255,7 @@
         <v>96</v>
       </c>
       <c r="D31">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="F31" s="1"/>
     </row>
@@ -5270,7 +5270,7 @@
         <v>97</v>
       </c>
       <c r="D32">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="F32" s="1"/>
     </row>
@@ -5393,7 +5393,7 @@
         <v>86</v>
       </c>
       <c r="D39">
-        <v>0.7</v>
+        <v>0.67</v>
       </c>
       <c r="E39" t="s">
         <v>106</v>
@@ -5411,7 +5411,7 @@
         <v>105</v>
       </c>
       <c r="D40">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="E40" t="s">
         <v>107</v>
@@ -5429,7 +5429,7 @@
         <v>87</v>
       </c>
       <c r="D41">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="E41" t="s">
         <v>108</v>
@@ -5539,7 +5539,7 @@
         <v>7</v>
       </c>
       <c r="D48">
-        <v>0.03</v>
+        <v>2.7E-2</v>
       </c>
       <c r="E48" t="s">
         <v>102</v>
@@ -5576,7 +5576,7 @@
         <v>139</v>
       </c>
       <c r="D50">
-        <v>0.3</v>
+        <v>0.33</v>
       </c>
       <c r="E50" t="s">
         <v>140</v>
@@ -5593,7 +5593,7 @@
         <v>142</v>
       </c>
       <c r="D51">
-        <v>2030</v>
+        <v>2028.5</v>
       </c>
       <c r="E51" t="s">
         <v>144</v>

</xml_diff>

<commit_message>
phi, eta read from scenario_params.xlsx
</commit_message>
<xml_diff>
--- a/inst/ext_data/scenario_parameters.xlsx
+++ b/inst/ext_data/scenario_parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\depmicrosimr\inst\ext_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A23481F8-ECA7-40B9-ABFB-40916E9786EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EF1C66B-DCF0-4D2F-94B6-7123E306D0B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Description" sheetId="7" r:id="rId1"/>
@@ -19,8 +19,10 @@
     <sheet name="LDSC" sheetId="18" r:id="rId4"/>
     <sheet name="LowPrice" sheetId="21" r:id="rId5"/>
     <sheet name="HighPrice" sheetId="19" r:id="rId6"/>
+    <sheet name="EDSC_sens" sheetId="22" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="993" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1224" uniqueCount="164">
   <si>
     <t>category</t>
   </si>
@@ -527,6 +529,30 @@
   </si>
   <si>
     <t>-50€ discount in 2030 and 2040</t>
+  </si>
+  <si>
+    <t>eta.</t>
+  </si>
+  <si>
+    <t>default inflexible fraction</t>
+  </si>
+  <si>
+    <t>default ramping cost</t>
+  </si>
+  <si>
+    <t>phi.</t>
+  </si>
+  <si>
+    <t>EDSC_sens</t>
+  </si>
+  <si>
+    <t>EDSC sensitiviy</t>
+  </si>
+  <si>
+    <t>varies phi and eta values</t>
+  </si>
+  <si>
+    <t>NB: MODEL RECALIBRATION REQUIRED</t>
   </si>
 </sst>
 </file>
@@ -652,7 +678,7 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -683,7 +709,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="4"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1005,7 +1030,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2536B528-ACE0-4AEE-80FE-2144BA4A4410}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="33.6" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.44140625" style="15" customWidth="1"/>
@@ -1016,7 +1041,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="18" t="s">
         <v>118</v>
       </c>
     </row>
@@ -1138,6 +1163,20 @@
       </c>
       <c r="B10" s="2" t="s">
         <v>151</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -1147,7 +1186,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C8E1679-ADB0-42D7-8103-5D0EB0C9F50E}">
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -2003,6 +2042,34 @@
         <v>124</v>
       </c>
     </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>6</v>
+      </c>
+      <c r="B50" t="s">
+        <v>158</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="D50">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>6</v>
+      </c>
+      <c r="B51" t="s">
+        <v>157</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="D51">
+        <v>0.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2010,7 +2077,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFE7130B-2B6C-40C3-A565-474237859EF4}">
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -2866,6 +2933,34 @@
         <v>124</v>
       </c>
     </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>6</v>
+      </c>
+      <c r="B50" t="s">
+        <v>158</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="D50">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>6</v>
+      </c>
+      <c r="B51" t="s">
+        <v>157</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="D51">
+        <v>0.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2873,7 +2968,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A8FF8BC-953A-45D1-A042-B3C357C0F4A0}">
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -3034,7 +3129,7 @@
       <c r="E9" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" t="s">
         <v>134</v>
       </c>
     </row>
@@ -3054,7 +3149,7 @@
       <c r="E10" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="18" t="s">
+      <c r="F10" t="s">
         <v>134</v>
       </c>
     </row>
@@ -3729,6 +3824,34 @@
       </c>
       <c r="E49" t="s">
         <v>124</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>6</v>
+      </c>
+      <c r="B50" t="s">
+        <v>158</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="D50">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>6</v>
+      </c>
+      <c r="B51" t="s">
+        <v>157</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="D51">
+        <v>0.4</v>
       </c>
     </row>
   </sheetData>
@@ -3738,7 +3861,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0BB0FBB-7CC2-42FB-B919-41F4158D78FF}">
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -4596,6 +4719,34 @@
         <v>124</v>
       </c>
     </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>6</v>
+      </c>
+      <c r="B50" t="s">
+        <v>158</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="D50">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>6</v>
+      </c>
+      <c r="B51" t="s">
+        <v>157</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="D51">
+        <v>0.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4603,7 +4754,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{637651EF-BBD1-4820-B575-600BCC8F4568}">
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.88671875" customWidth="1"/>
@@ -5459,6 +5610,925 @@
         <v>124</v>
       </c>
     </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>6</v>
+      </c>
+      <c r="B50" t="s">
+        <v>158</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="D50">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>6</v>
+      </c>
+      <c r="B51" t="s">
+        <v>157</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="D51">
+        <v>0.4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2769E098-C0F9-4DD7-9574-53532E344D3F}">
+  <dimension ref="A1:F51"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="2" max="2" width="41.88671875" customWidth="1"/>
+    <col min="3" max="3" width="55" customWidth="1"/>
+    <col min="4" max="4" width="16.5546875" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" customWidth="1"/>
+    <col min="6" max="6" width="22.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2">
+        <v>2026.5</v>
+      </c>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3">
+        <v>2021</v>
+      </c>
+      <c r="F3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4">
+        <v>0.13500000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D5">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D6">
+        <v>0.13500000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>111</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="D7">
+        <v>0.5</v>
+      </c>
+      <c r="E7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>69</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D8" s="17">
+        <v>9.2999999999999999E-2</v>
+      </c>
+      <c r="E8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" s="17">
+        <v>0.1</v>
+      </c>
+      <c r="E9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" s="17">
+        <v>0.1</v>
+      </c>
+      <c r="E10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="7">
+        <v>0.16838500000000001</v>
+      </c>
+      <c r="E11" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="7">
+        <v>7.2419999999999998E-2</v>
+      </c>
+      <c r="E12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="7">
+        <v>0.19167500000000001</v>
+      </c>
+      <c r="E13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14">
+        <v>0.1981</v>
+      </c>
+      <c r="E14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15">
+        <v>8.5199999999999998E-2</v>
+      </c>
+      <c r="E15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16">
+        <v>0.22550000000000001</v>
+      </c>
+      <c r="E16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" s="7">
+        <v>0.21791000000000002</v>
+      </c>
+      <c r="E17" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="D18" s="7">
+        <v>0.10501000000000002</v>
+      </c>
+      <c r="E18" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18" s="7">
+        <f>D17-D14</f>
+        <v>1.9810000000000022E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D19" s="7">
+        <v>0.24531000000000003</v>
+      </c>
+      <c r="E19" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D20" s="7">
+        <v>0.25752999999999998</v>
+      </c>
+      <c r="E20" t="s">
+        <v>15</v>
+      </c>
+      <c r="F20" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" t="s">
+        <v>34</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D21" s="7">
+        <v>0.14462999999999998</v>
+      </c>
+      <c r="E21" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" s="7">
+        <f>(D20-D14)</f>
+        <v>5.9429999999999983E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="D22" s="7">
+        <v>0.28493000000000002</v>
+      </c>
+      <c r="E22" t="s">
+        <v>15</v>
+      </c>
+      <c r="F22" s="7"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>14</v>
+      </c>
+      <c r="B23" t="s">
+        <v>19</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23">
+        <v>130</v>
+      </c>
+      <c r="E23" t="s">
+        <v>21</v>
+      </c>
+      <c r="F23" s="1"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>14</v>
+      </c>
+      <c r="B24" t="s">
+        <v>26</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D24">
+        <v>215</v>
+      </c>
+      <c r="F24" s="1"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B25" t="s">
+        <v>27</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D25">
+        <v>265</v>
+      </c>
+      <c r="F25" s="1"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B26" t="s">
+        <v>28</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D26">
+        <v>320</v>
+      </c>
+      <c r="F26" s="1"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B27" t="s">
+        <v>29</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D27">
+        <v>350</v>
+      </c>
+      <c r="F27" s="1"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28" t="s">
+        <v>67</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="D28" s="17">
+        <v>75</v>
+      </c>
+      <c r="F28" s="1"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>14</v>
+      </c>
+      <c r="B29" t="s">
+        <v>65</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D29" s="17">
+        <v>0</v>
+      </c>
+      <c r="F29" s="1"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>14</v>
+      </c>
+      <c r="B30" t="s">
+        <v>66</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="D30" s="17">
+        <v>0</v>
+      </c>
+      <c r="F30" s="1"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" t="s">
+        <v>62</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="D31">
+        <v>12</v>
+      </c>
+      <c r="E31" t="s">
+        <v>64</v>
+      </c>
+      <c r="F31" s="1"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>72</v>
+      </c>
+      <c r="B32" t="s">
+        <v>75</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D32">
+        <v>0.88</v>
+      </c>
+      <c r="E32" t="s">
+        <v>72</v>
+      </c>
+      <c r="F32" s="1"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>72</v>
+      </c>
+      <c r="B33" t="s">
+        <v>76</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="D33">
+        <v>0.88</v>
+      </c>
+      <c r="E33" t="s">
+        <v>72</v>
+      </c>
+      <c r="F33" s="1"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>72</v>
+      </c>
+      <c r="B34" t="s">
+        <v>83</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="D34">
+        <v>2.25</v>
+      </c>
+      <c r="E34" t="s">
+        <v>128</v>
+      </c>
+      <c r="F34" s="1"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>72</v>
+      </c>
+      <c r="B35" t="s">
+        <v>77</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="D35">
+        <v>0.61</v>
+      </c>
+      <c r="E35" t="s">
+        <v>72</v>
+      </c>
+      <c r="F35" s="1"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>72</v>
+      </c>
+      <c r="B36" t="s">
+        <v>77</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D36">
+        <v>0.69</v>
+      </c>
+      <c r="E36" t="s">
+        <v>72</v>
+      </c>
+      <c r="F36" s="1"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>72</v>
+      </c>
+      <c r="B37" t="s">
+        <v>78</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="D37">
+        <v>0.65</v>
+      </c>
+      <c r="E37" t="s">
+        <v>99</v>
+      </c>
+      <c r="F37" s="1"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>72</v>
+      </c>
+      <c r="B38" t="s">
+        <v>97</v>
+      </c>
+      <c r="C38" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="D38">
+        <v>0.85</v>
+      </c>
+      <c r="E38" t="s">
+        <v>100</v>
+      </c>
+      <c r="F38" s="1"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>72</v>
+      </c>
+      <c r="B39" t="s">
+        <v>79</v>
+      </c>
+      <c r="C39" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="D39">
+        <v>0.4</v>
+      </c>
+      <c r="E39" t="s">
+        <v>101</v>
+      </c>
+      <c r="F39" s="1"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>72</v>
+      </c>
+      <c r="B40" t="s">
+        <v>102</v>
+      </c>
+      <c r="C40" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="D40">
+        <v>4.25</v>
+      </c>
+      <c r="F40" s="1"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>72</v>
+      </c>
+      <c r="B41" t="s">
+        <v>104</v>
+      </c>
+      <c r="C41" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="D41">
+        <v>1.25</v>
+      </c>
+      <c r="F41" s="1"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>6</v>
+      </c>
+      <c r="B42" t="s">
+        <v>106</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>6</v>
+      </c>
+      <c r="B43" t="s">
+        <v>107</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D43">
+        <v>2</v>
+      </c>
+      <c r="F43" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>6</v>
+      </c>
+      <c r="B44" t="s">
+        <v>106</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="D44">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>6</v>
+      </c>
+      <c r="B45" t="s">
+        <v>107</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D45">
+        <v>4</v>
+      </c>
+      <c r="F45" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>6</v>
+      </c>
+      <c r="B46" t="s">
+        <v>93</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D46">
+        <v>3.3000000000000002E-2</v>
+      </c>
+      <c r="E46" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>6</v>
+      </c>
+      <c r="B47" t="s">
+        <v>30</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D47">
+        <v>0.01</v>
+      </c>
+      <c r="E47" t="s">
+        <v>31</v>
+      </c>
+      <c r="F47" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>6</v>
+      </c>
+      <c r="B48" t="s">
+        <v>86</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D48">
+        <v>0.33</v>
+      </c>
+      <c r="E48" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>6</v>
+      </c>
+      <c r="B49" t="s">
+        <v>123</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D49">
+        <v>2028.5</v>
+      </c>
+      <c r="E49" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>6</v>
+      </c>
+      <c r="B50" t="s">
+        <v>158</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="D50">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>6</v>
+      </c>
+      <c r="B51" t="s">
+        <v>157</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="D51">
+        <v>0.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
hindsight version set as default. Use v1.80 for foresight version
</commit_message>
<xml_diff>
--- a/inst/ext_data/scenario_parameters.xlsx
+++ b/inst/ext_data/scenario_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\depmicrosimr\inst\ext_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EF1C66B-DCF0-4D2F-94B6-7123E306D0B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F774B42E-9879-48AA-BBE4-FFB19EAE9C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,6 @@
     <sheet name="EDSC_sens" sheetId="22" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -6295,7 +6294,7 @@
         <v>81</v>
       </c>
       <c r="D37">
-        <v>0.65</v>
+        <v>0.7</v>
       </c>
       <c r="E37" t="s">
         <v>99</v>
@@ -6313,7 +6312,7 @@
         <v>98</v>
       </c>
       <c r="D38">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="E38" t="s">
         <v>100</v>
@@ -6331,7 +6330,7 @@
         <v>82</v>
       </c>
       <c r="D39">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="E39" t="s">
         <v>101</v>
@@ -6478,7 +6477,7 @@
         <v>120</v>
       </c>
       <c r="D48">
-        <v>0.33</v>
+        <v>0.24</v>
       </c>
       <c r="E48" t="s">
         <v>121</v>

</xml_diff>

<commit_message>
foresight TRUE or FALSE added to scenario_parameters
</commit_message>
<xml_diff>
--- a/inst/ext_data/scenario_parameters.xlsx
+++ b/inst/ext_data/scenario_parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\depmicrosimr\inst\ext_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F774B42E-9879-48AA-BBE4-FFB19EAE9C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{370D953B-A751-457A-81BF-D139A56D8417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Description" sheetId="7" r:id="rId1"/>
@@ -19,9 +19,9 @@
     <sheet name="LDSC" sheetId="18" r:id="rId4"/>
     <sheet name="LowPrice" sheetId="21" r:id="rId5"/>
     <sheet name="HighPrice" sheetId="19" r:id="rId6"/>
-    <sheet name="EDSC_sens" sheetId="22" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1224" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="167">
   <si>
     <t>category</t>
   </si>
@@ -416,9 +416,6 @@
     <t>random battery uptake model means that flex_score distribution become right-skewed</t>
   </si>
   <si>
-    <t>depmicromsimr scenario descriptions</t>
-  </si>
-  <si>
     <t>label</t>
   </si>
   <si>
@@ -552,6 +549,18 @@
   </si>
   <si>
     <t>NB: MODEL RECALIBRATION REQUIRED</t>
+  </si>
+  <si>
+    <t>flex reward withheld</t>
+  </si>
+  <si>
+    <t>depmicromsimr scenario descriptions - foresight</t>
+  </si>
+  <si>
+    <t>foresight</t>
+  </si>
+  <si>
+    <t>calibration based on perfect foresight if TRUE or perfect hindisght if FALSE</t>
   </si>
 </sst>
 </file>
@@ -709,7 +718,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="4"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -1041,12 +1050,12 @@
   <sheetData>
     <row r="1" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="18" t="s">
-        <v>118</v>
+        <v>164</v>
       </c>
     </row>
     <row r="2" spans="1:4" s="4" customFormat="1" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>9</v>
@@ -1063,27 +1072,27 @@
         <v>94</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C3" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>131</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1091,13 +1100,13 @@
         <v>112</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1105,13 +1114,13 @@
         <v>113</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1119,13 +1128,13 @@
         <v>114</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>140</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1133,13 +1142,13 @@
         <v>115</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1147,10 +1156,10 @@
         <v>116</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>117</v>
@@ -1158,24 +1167,24 @@
     </row>
     <row r="10" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="15" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>162</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -1185,7 +1194,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C8E1679-ADB0-42D7-8103-5D0EB0C9F50E}">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -1298,7 +1307,7 @@
         <v>111</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D7">
         <v>0.5</v>
@@ -1551,7 +1560,7 @@
         <v>15</v>
       </c>
       <c r="F20" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -1784,7 +1793,7 @@
         <v>2.25</v>
       </c>
       <c r="E34" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F34" s="1"/>
     </row>
@@ -2012,16 +2021,16 @@
         <v>6</v>
       </c>
       <c r="B48" t="s">
-        <v>86</v>
+        <v>163</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D48">
         <v>0.33</v>
       </c>
       <c r="E48" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
@@ -2029,16 +2038,16 @@
         <v>6</v>
       </c>
       <c r="B49" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D49">
         <v>2028.5</v>
       </c>
       <c r="E49" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
@@ -2046,10 +2055,10 @@
         <v>6</v>
       </c>
       <c r="B50" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D50">
         <v>0.3</v>
@@ -2060,13 +2069,30 @@
         <v>6</v>
       </c>
       <c r="B51" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D51">
         <v>0.4</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>6</v>
+      </c>
+      <c r="B52" t="s">
+        <v>165</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="D52">
+        <v>1</v>
+      </c>
+      <c r="E52" t="s">
+        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -2076,7 +2102,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFE7130B-2B6C-40C3-A565-474237859EF4}">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -2189,7 +2215,7 @@
         <v>111</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D7">
         <v>0.5</v>
@@ -2442,7 +2468,7 @@
         <v>15</v>
       </c>
       <c r="F20" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -2675,7 +2701,7 @@
         <v>2.25</v>
       </c>
       <c r="E34" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F34" s="1"/>
     </row>
@@ -2903,16 +2929,16 @@
         <v>6</v>
       </c>
       <c r="B48" t="s">
-        <v>86</v>
+        <v>163</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D48">
         <v>0.33</v>
       </c>
       <c r="E48" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
@@ -2920,16 +2946,16 @@
         <v>6</v>
       </c>
       <c r="B49" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D49">
         <v>2028.5</v>
       </c>
       <c r="E49" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
@@ -2937,10 +2963,10 @@
         <v>6</v>
       </c>
       <c r="B50" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D50">
         <v>0.3</v>
@@ -2951,13 +2977,30 @@
         <v>6</v>
       </c>
       <c r="B51" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D51">
         <v>0.4</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>6</v>
+      </c>
+      <c r="B52" t="s">
+        <v>165</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="D52">
+        <v>1</v>
+      </c>
+      <c r="E52" t="s">
+        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -2967,7 +3010,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A8FF8BC-953A-45D1-A042-B3C357C0F4A0}">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -3080,7 +3123,7 @@
         <v>111</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D7">
         <v>0.5</v>
@@ -3129,7 +3172,7 @@
         <v>15</v>
       </c>
       <c r="F9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -3149,7 +3192,7 @@
         <v>15</v>
       </c>
       <c r="F10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -3335,7 +3378,7 @@
         <v>15</v>
       </c>
       <c r="F20" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -3568,7 +3611,7 @@
         <v>2.25</v>
       </c>
       <c r="E34" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F34" s="1"/>
     </row>
@@ -3796,16 +3839,16 @@
         <v>6</v>
       </c>
       <c r="B48" t="s">
-        <v>86</v>
+        <v>163</v>
       </c>
       <c r="C48" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="D48">
+        <v>0.33</v>
+      </c>
+      <c r="E48" t="s">
         <v>120</v>
-      </c>
-      <c r="D48">
-        <v>3.3000000000000002E-2</v>
-      </c>
-      <c r="E48" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
@@ -3813,16 +3856,16 @@
         <v>6</v>
       </c>
       <c r="B49" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D49">
         <v>2028.5</v>
       </c>
       <c r="E49" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
@@ -3830,10 +3873,10 @@
         <v>6</v>
       </c>
       <c r="B50" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D50">
         <v>0.3</v>
@@ -3844,13 +3887,30 @@
         <v>6</v>
       </c>
       <c r="B51" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D51">
         <v>0.4</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>6</v>
+      </c>
+      <c r="B52" t="s">
+        <v>165</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="D52">
+        <v>1</v>
+      </c>
+      <c r="E52" t="s">
+        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -3860,7 +3920,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0BB0FBB-7CC2-42FB-B919-41F4158D78FF}">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -3973,7 +4033,7 @@
         <v>111</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D7">
         <v>0.5</v>
@@ -4022,7 +4082,7 @@
         <v>15</v>
       </c>
       <c r="F9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -4042,7 +4102,7 @@
         <v>15</v>
       </c>
       <c r="F10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -4228,7 +4288,7 @@
         <v>15</v>
       </c>
       <c r="F20" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -4461,7 +4521,7 @@
         <v>2.25</v>
       </c>
       <c r="E34" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F34" s="1"/>
     </row>
@@ -4689,16 +4749,16 @@
         <v>6</v>
       </c>
       <c r="B48" t="s">
-        <v>86</v>
+        <v>163</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D48">
         <v>0.33</v>
       </c>
       <c r="E48" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
@@ -4706,16 +4766,16 @@
         <v>6</v>
       </c>
       <c r="B49" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D49">
         <v>2028.5</v>
       </c>
       <c r="E49" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
@@ -4723,10 +4783,10 @@
         <v>6</v>
       </c>
       <c r="B50" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D50">
         <v>0.3</v>
@@ -4737,13 +4797,30 @@
         <v>6</v>
       </c>
       <c r="B51" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D51">
         <v>0.4</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>6</v>
+      </c>
+      <c r="B52" t="s">
+        <v>165</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="D52">
+        <v>1</v>
+      </c>
+      <c r="E52" t="s">
+        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -4753,7 +4830,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{637651EF-BBD1-4820-B575-600BCC8F4568}">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.88671875" customWidth="1"/>
@@ -4864,7 +4941,7 @@
         <v>111</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D7">
         <v>0.5</v>
@@ -4913,7 +4990,7 @@
         <v>15</v>
       </c>
       <c r="F9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -4933,7 +5010,7 @@
         <v>15</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -5119,7 +5196,7 @@
         <v>15</v>
       </c>
       <c r="F20" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -5352,7 +5429,7 @@
         <v>2.25</v>
       </c>
       <c r="E34" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F34" s="1"/>
     </row>
@@ -5583,13 +5660,13 @@
         <v>86</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D48">
         <v>3.3000000000000002E-2</v>
       </c>
       <c r="E48" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
@@ -5597,16 +5674,16 @@
         <v>6</v>
       </c>
       <c r="B49" t="s">
-        <v>123</v>
+        <v>163</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D49">
         <v>2028.5</v>
       </c>
       <c r="E49" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
@@ -5614,10 +5691,10 @@
         <v>6</v>
       </c>
       <c r="B50" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D50">
         <v>0.3</v>
@@ -5628,904 +5705,30 @@
         <v>6</v>
       </c>
       <c r="B51" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D51">
         <v>0.4</v>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2769E098-C0F9-4DD7-9574-53532E344D3F}">
-  <dimension ref="A1:F51"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="2" max="2" width="41.88671875" customWidth="1"/>
-    <col min="3" max="3" width="55" customWidth="1"/>
-    <col min="4" max="4" width="16.5546875" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" customWidth="1"/>
-    <col min="6" max="6" width="22.5546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>6</v>
+      </c>
+      <c r="B52" t="s">
+        <v>165</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="D52">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2">
-        <v>2026.5</v>
-      </c>
-      <c r="F2" s="1"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3">
-        <v>2021</v>
-      </c>
-      <c r="F3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="D4">
-        <v>0.13500000000000001</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>57</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D5">
-        <v>0.09</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" t="s">
-        <v>60</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="D6">
-        <v>0.13500000000000001</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>111</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="D7">
-        <v>0.5</v>
-      </c>
-      <c r="E7" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="D8" s="17">
-        <v>9.2999999999999999E-2</v>
-      </c>
-      <c r="E8" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" t="s">
-        <v>52</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D9" s="17">
-        <v>0.1</v>
-      </c>
-      <c r="E9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" t="s">
-        <v>53</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="D10" s="17">
-        <v>0.1</v>
-      </c>
-      <c r="E10" t="s">
-        <v>15</v>
-      </c>
-      <c r="F10" s="1"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D11" s="7">
-        <v>0.16838500000000001</v>
-      </c>
-      <c r="E11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F11" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" t="s">
-        <v>34</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="D12" s="7">
-        <v>7.2419999999999998E-2</v>
-      </c>
-      <c r="E12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="D13" s="7">
-        <v>0.19167500000000001</v>
-      </c>
-      <c r="E13" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="D14">
-        <v>0.1981</v>
-      </c>
-      <c r="E14" t="s">
-        <v>15</v>
-      </c>
-      <c r="F14" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15" t="s">
-        <v>34</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="D15">
-        <v>8.5199999999999998E-2</v>
-      </c>
-      <c r="E15" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="D16">
-        <v>0.22550000000000001</v>
-      </c>
-      <c r="E16" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D17" s="7">
-        <v>0.21791000000000002</v>
-      </c>
-      <c r="E17" t="s">
-        <v>15</v>
-      </c>
-      <c r="F17" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>14</v>
-      </c>
-      <c r="B18" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="D18" s="7">
-        <v>0.10501000000000002</v>
-      </c>
-      <c r="E18" t="s">
-        <v>15</v>
-      </c>
-      <c r="F18" s="7">
-        <f>D17-D14</f>
-        <v>1.9810000000000022E-2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C19" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D19" s="7">
-        <v>0.24531000000000003</v>
-      </c>
-      <c r="E19" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="D20" s="7">
-        <v>0.25752999999999998</v>
-      </c>
-      <c r="E20" t="s">
-        <v>15</v>
-      </c>
-      <c r="F20" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>14</v>
-      </c>
-      <c r="B21" t="s">
-        <v>34</v>
-      </c>
-      <c r="C21" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="D21" s="7">
-        <v>0.14462999999999998</v>
-      </c>
-      <c r="E21" t="s">
-        <v>15</v>
-      </c>
-      <c r="F21" s="7">
-        <f>(D20-D14)</f>
-        <v>5.9429999999999983E-2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C22" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="D22" s="7">
-        <v>0.28493000000000002</v>
-      </c>
-      <c r="E22" t="s">
-        <v>15</v>
-      </c>
-      <c r="F22" s="7"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>14</v>
-      </c>
-      <c r="B23" t="s">
-        <v>19</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D23">
-        <v>130</v>
-      </c>
-      <c r="E23" t="s">
-        <v>21</v>
-      </c>
-      <c r="F23" s="1"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>14</v>
-      </c>
-      <c r="B24" t="s">
-        <v>26</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D24">
-        <v>215</v>
-      </c>
-      <c r="F24" s="1"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>14</v>
-      </c>
-      <c r="B25" t="s">
-        <v>27</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D25">
-        <v>265</v>
-      </c>
-      <c r="F25" s="1"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>14</v>
-      </c>
-      <c r="B26" t="s">
-        <v>28</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D26">
-        <v>320</v>
-      </c>
-      <c r="F26" s="1"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>14</v>
-      </c>
-      <c r="B27" t="s">
-        <v>29</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D27">
-        <v>350</v>
-      </c>
-      <c r="F27" s="1"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>14</v>
-      </c>
-      <c r="B28" t="s">
-        <v>67</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="D28" s="17">
-        <v>75</v>
-      </c>
-      <c r="F28" s="1"/>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>14</v>
-      </c>
-      <c r="B29" t="s">
-        <v>65</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="D29" s="17">
-        <v>0</v>
-      </c>
-      <c r="F29" s="1"/>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>14</v>
-      </c>
-      <c r="B30" t="s">
-        <v>66</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="D30" s="17">
-        <v>0</v>
-      </c>
-      <c r="F30" s="1"/>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>33</v>
-      </c>
-      <c r="B31" t="s">
-        <v>62</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="D31">
-        <v>12</v>
-      </c>
-      <c r="E31" t="s">
-        <v>64</v>
-      </c>
-      <c r="F31" s="1"/>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>72</v>
-      </c>
-      <c r="B32" t="s">
-        <v>75</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="D32">
-        <v>0.88</v>
-      </c>
-      <c r="E32" t="s">
-        <v>72</v>
-      </c>
-      <c r="F32" s="1"/>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>72</v>
-      </c>
-      <c r="B33" t="s">
-        <v>76</v>
-      </c>
-      <c r="C33" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="D33">
-        <v>0.88</v>
-      </c>
-      <c r="E33" t="s">
-        <v>72</v>
-      </c>
-      <c r="F33" s="1"/>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>72</v>
-      </c>
-      <c r="B34" t="s">
-        <v>83</v>
-      </c>
-      <c r="C34" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="D34">
-        <v>2.25</v>
-      </c>
-      <c r="E34" t="s">
-        <v>128</v>
-      </c>
-      <c r="F34" s="1"/>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>72</v>
-      </c>
-      <c r="B35" t="s">
-        <v>77</v>
-      </c>
-      <c r="C35" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="D35">
-        <v>0.61</v>
-      </c>
-      <c r="E35" t="s">
-        <v>72</v>
-      </c>
-      <c r="F35" s="1"/>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>72</v>
-      </c>
-      <c r="B36" t="s">
-        <v>77</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>85</v>
-      </c>
-      <c r="D36">
-        <v>0.69</v>
-      </c>
-      <c r="E36" t="s">
-        <v>72</v>
-      </c>
-      <c r="F36" s="1"/>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>72</v>
-      </c>
-      <c r="B37" t="s">
-        <v>78</v>
-      </c>
-      <c r="C37" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="D37">
-        <v>0.7</v>
-      </c>
-      <c r="E37" t="s">
-        <v>99</v>
-      </c>
-      <c r="F37" s="1"/>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>72</v>
-      </c>
-      <c r="B38" t="s">
-        <v>97</v>
-      </c>
-      <c r="C38" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="D38">
-        <v>0.9</v>
-      </c>
-      <c r="E38" t="s">
-        <v>100</v>
-      </c>
-      <c r="F38" s="1"/>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>72</v>
-      </c>
-      <c r="B39" t="s">
-        <v>79</v>
-      </c>
-      <c r="C39" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="D39">
-        <v>0.45</v>
-      </c>
-      <c r="E39" t="s">
-        <v>101</v>
-      </c>
-      <c r="F39" s="1"/>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>72</v>
-      </c>
-      <c r="B40" t="s">
-        <v>102</v>
-      </c>
-      <c r="C40" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="D40">
-        <v>4.25</v>
-      </c>
-      <c r="F40" s="1"/>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>72</v>
-      </c>
-      <c r="B41" t="s">
-        <v>104</v>
-      </c>
-      <c r="C41" s="13" t="s">
-        <v>105</v>
-      </c>
-      <c r="D41">
-        <v>1.25</v>
-      </c>
-      <c r="F41" s="1"/>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
-        <v>6</v>
-      </c>
-      <c r="B42" t="s">
-        <v>106</v>
-      </c>
-      <c r="C42" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="D42">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
-        <v>6</v>
-      </c>
-      <c r="B43" t="s">
-        <v>107</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="D43">
-        <v>2</v>
-      </c>
-      <c r="F43" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
-        <v>6</v>
-      </c>
-      <c r="B44" t="s">
-        <v>106</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="D44">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>6</v>
-      </c>
-      <c r="B45" t="s">
-        <v>107</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="D45">
-        <v>4</v>
-      </c>
-      <c r="F45" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" t="s">
-        <v>6</v>
-      </c>
-      <c r="B46" t="s">
-        <v>93</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D46">
-        <v>3.3000000000000002E-2</v>
-      </c>
-      <c r="E46" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
-        <v>6</v>
-      </c>
-      <c r="B47" t="s">
-        <v>30</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D47">
-        <v>0.01</v>
-      </c>
-      <c r="E47" t="s">
-        <v>31</v>
-      </c>
-      <c r="F47" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" t="s">
-        <v>6</v>
-      </c>
-      <c r="B48" t="s">
-        <v>86</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="D48">
-        <v>0.24</v>
-      </c>
-      <c r="E48" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
-        <v>6</v>
-      </c>
-      <c r="B49" t="s">
-        <v>123</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="D49">
-        <v>2028.5</v>
-      </c>
-      <c r="E49" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
-        <v>6</v>
-      </c>
-      <c r="B50" t="s">
-        <v>158</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="D50">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
-        <v>6</v>
-      </c>
-      <c r="B51" t="s">
-        <v>157</v>
-      </c>
-      <c r="C51" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="D51">
-        <v>0.6</v>
+      <c r="E52" t="s">
+        <v>166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
parameter bug fix in highprice scenario
</commit_message>
<xml_diff>
--- a/inst/ext_data/scenario_parameters.xlsx
+++ b/inst/ext_data/scenario_parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\depmicrosimr\inst\ext_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{370D953B-A751-457A-81BF-D139A56D8417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1256F0E1-F530-4A9E-96A0-B56DFC2F56B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Description" sheetId="7" r:id="rId1"/>
@@ -21,7 +21,6 @@
     <sheet name="HighPrice" sheetId="19" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -554,13 +553,13 @@
     <t>flex reward withheld</t>
   </si>
   <si>
-    <t>depmicromsimr scenario descriptions - foresight</t>
-  </si>
-  <si>
     <t>foresight</t>
   </si>
   <si>
     <t>calibration based on perfect foresight if TRUE or perfect hindisght if FALSE</t>
+  </si>
+  <si>
+    <t>depmicromsimr scenario descriptions - default</t>
   </si>
 </sst>
 </file>
@@ -1050,7 +1049,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="18" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2" spans="1:4" s="4" customFormat="1" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2083,16 +2082,16 @@
         <v>6</v>
       </c>
       <c r="B52" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D52">
         <v>1</v>
       </c>
       <c r="E52" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -2991,16 +2990,16 @@
         <v>6</v>
       </c>
       <c r="B52" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D52">
         <v>1</v>
       </c>
       <c r="E52" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -3901,16 +3900,16 @@
         <v>6</v>
       </c>
       <c r="B52" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D52">
         <v>1</v>
       </c>
       <c r="E52" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -4811,16 +4810,16 @@
         <v>6</v>
       </c>
       <c r="B52" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D52">
         <v>1</v>
       </c>
       <c r="E52" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -5663,7 +5662,7 @@
         <v>119</v>
       </c>
       <c r="D48">
-        <v>3.3000000000000002E-2</v>
+        <v>0.33</v>
       </c>
       <c r="E48" t="s">
         <v>120</v>
@@ -5719,16 +5718,16 @@
         <v>6</v>
       </c>
       <c r="B52" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D52">
         <v>1</v>
       </c>
       <c r="E52" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>